<commit_message>
Make FSLR framework active build
</commit_message>
<xml_diff>
--- a/outputs/first_solar_fslr_research_workbook.xlsx
+++ b/outputs/first_solar_fslr_research_workbook.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Raee92c6bd788473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials KPIs" sheetId="2" r:id="R5986b72791b842e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="3" r:id="Red943189d442493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="4" r:id="Rd6ac2b3e4164475d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Reaction" sheetId="5" r:id="Ra44439fdaf8a48a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts Policy Risks" sheetId="6" r:id="Rdcb6f1501b1149cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Path" sheetId="7" r:id="R17dc5d9a6b734a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R780936637bcc41fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" r:id="R4b40306d70af4667"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Raa3e350abe064267"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials KPIs" sheetId="2" r:id="R7ac5dcd0eb514b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="3" r:id="R488457ed4eda460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="4" r:id="R19ec32e1e61e4601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Reaction" sheetId="5" r:id="Rdbd34a3554bf4deb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts Policy Risks" sheetId="6" r:id="Rb837ce83d78b4803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Path" sheetId="7" r:id="R8d73575ec81d449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Framework" sheetId="8" r:id="R0be13a1b9d484910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Re3cd0fa476624434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" r:id="R00d4e8174d3749bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -910,7 +911,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra2c584db0cef43d2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R72faadc990244cbd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -940,7 +941,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7c3add9e18114ab3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec4cd7f896dc4463"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -975,7 +976,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R14a6b54ca68f4a11"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra168798b763b4dda"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1010,7 +1011,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R69b7dcec84d74e63"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R376a667b43c446f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1045,7 +1046,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b7056e847194a5c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rff965926c230474e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1126,8 +1127,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CatalystsTable" displayName="CatalystsTable" ref="A4:H10" headerRowCount="1">
-  <x:autoFilter ref="A4:H10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CatalystsTable" displayName="CatalystsTable" ref="A4:H11" headerRowCount="1">
+  <x:autoFilter ref="A4:H11"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="date_or_window"/>
     <x:tableColumn id="2" name="category"/>
@@ -1158,7 +1159,22 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="SourcesTable" displayName="SourcesTable" ref="A4:H18" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ActionFrameworkTable" displayName="ActionFrameworkTable" ref="A4:F10" headerRowCount="1">
+  <x:autoFilter ref="A4:F10"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="action"/>
+    <x:tableColumn id="2" name="price_zone"/>
+    <x:tableColumn id="3" name="position_action"/>
+    <x:tableColumn id="4" name="operating_triggers"/>
+    <x:tableColumn id="5" name="risk_control"/>
+    <x:tableColumn id="6" name="source_id"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourcesTable" displayName="SourcesTable" ref="A4:H18" headerRowCount="1">
   <x:autoFilter ref="A4:H18"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="source_id"/>
@@ -1422,7 +1438,7 @@
         <x:v>投资方向</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>已有仓位继续跟踪；新资金等待回撤或订单/政策验证后分批</x:v>
+        <x:v>当前价格附近偏买/主动建仓；不是深度低估，但 $290-$310 区间风险收益足够做初始仓位</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
@@ -1445,10 +1461,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
-        <x:v>当前股价</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="n">
-        <x:v>289.495</x:v>
+        <x:v>建仓/加仓</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>$290-$310 建 40%-60% 目标仓位；$260-$280 且 thesis intact 加；$310-$330 只为经营确认加</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2" t="str">
@@ -1471,11 +1487,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="str">
-        <x:v>公司口径 EV</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="n">
-        <x:f>Valuation!B9</x:f>
-        <x:v>29.153178425</x:v>
+        <x:v>减仓/认错</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>$360-$380 无经营上修则减仓；&lt;$250-$255 且 thesis break，或经营触发器失效，则减至小仓/退出</x:v>
       </x:c>
       <x:c r="C7" s="2"/>
       <x:c r="D7" s="2" t="str">
@@ -1498,11 +1513,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>EV/FY2026 EBITDA</x:v>
-      </x:c>
-      <x:c r="B8" s="10" t="n">
-        <x:f>Valuation!B15</x:f>
-        <x:v>10.79747349074074</x:v>
+        <x:v>当前股价</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="n">
+        <x:v>294.41</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="2" t="str">
@@ -1525,11 +1539,11 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>TTM P/E</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="n">
-        <x:f>Valuation!B13</x:f>
-        <x:v>18.701227390180875</x:v>
+        <x:v>公司口径 EV</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="n">
+        <x:f>Valuation!B9</x:f>
+        <x:v>29.68210615</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
@@ -1546,10 +1560,11 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>Backlog</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="str">
-        <x:v>47.9GW / $14.4bn</x:v>
+        <x:v>EV/FY2026 EBITDA</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="n">
+        <x:f>Valuation!B15</x:f>
+        <x:v>10.993372648148148</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -1566,11 +1581,11 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>Backlog ASP</x:v>
-      </x:c>
-      <x:c r="B11" s="11" t="n">
-        <x:f>Valuation!B18</x:f>
-        <x:v>0.3006263048016702</x:v>
+        <x:v>TTM P/E</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="n">
+        <x:f>Valuation!B13</x:f>
+        <x:v>19.0187338501292</x:v>
       </x:c>
       <x:c r="C11" s="2"/>
       <x:c r="D11" s="2"/>
@@ -1587,10 +1602,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
-        <x:v>最关键问题</x:v>
+        <x:v>Backlog</x:v>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>45X 和贸易政策能否把 backlog 变成 2027+ 可持续现金流</x:v>
+        <x:v>47.9GW / $14.4bn</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="13" t="str">
@@ -1613,10 +1628,11 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="str">
-        <x:v>下一步验证</x:v>
-      </x:c>
-      <x:c r="B13" s="2" t="str">
-        <x:v>新增 bookings ASP、45X cash realization、OCF-capex、Section 232/TOPCon</x:v>
+        <x:v>Backlog ASP</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="n">
+        <x:f>Valuation!B18</x:f>
+        <x:v>0.3006263048016702</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2" t="str">
@@ -1627,7 +1643,7 @@
       </x:c>
       <x:c r="F13" s="16" t="n">
         <x:f>E13/Valuation!$B$5-1</x:f>
-        <x:v>-0.345161998384097</x:v>
+        <x:v>-0.35609412969058174</x:v>
       </x:c>
       <x:c r="G13" s="2"/>
       <x:c r="H13" s="2"/>
@@ -1640,10 +1656,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="str">
-        <x:v>资料路径</x:v>
+        <x:v>最关键问题</x:v>
       </x:c>
       <x:c r="B14" s="2" t="str">
-        <x:v>见 Sources sheet 和 data/sources.csv</x:v>
+        <x:v>45X 和贸易政策能否把 backlog 变成 2027+ 可持续现金流</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
       <x:c r="D14" s="2" t="str">
@@ -1654,7 +1670,7 @@
       </x:c>
       <x:c r="F14" s="16" t="n">
         <x:f>E14/Valuation!$B$5-1</x:f>
-        <x:v>-0.06911401807698747</x:v>
+        <x:v>-0.08465460637613365</x:v>
       </x:c>
       <x:c r="G14" s="2"/>
       <x:c r="H14" s="2"/>
@@ -1666,19 +1682,2389 @@
       <x:c r="N14" s="2"/>
     </x:row>
     <x:row r="15">
+      <x:c r="A15" s="2" t="str">
+        <x:v>下一步验证</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>新增 bookings ASP、45X cash realization、OCF-capex、Section 232/TOPCon</x:v>
+      </x:c>
+      <x:c r="C15" s="2"/>
+      <x:c r="D15" s="2" t="str">
+        <x:v>Bull</x:v>
+      </x:c>
+      <x:c r="E15" s="15" t="n">
+        <x:v>375.4200250894393</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="n">
+        <x:f>E15/Valuation!$B$5-1</x:f>
+        <x:v>0.2751605756918558</x:v>
+      </x:c>
+      <x:c r="G15" s="2"/>
+      <x:c r="H15" s="2"/>
+      <x:c r="I15" s="2"/>
+      <x:c r="J15" s="2"/>
+      <x:c r="K15" s="2"/>
+      <x:c r="L15" s="2"/>
+      <x:c r="M15" s="2"/>
+      <x:c r="N15" s="2"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
+        <x:v>资料路径</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>见 Sources sheet 和 data/sources.csv</x:v>
+      </x:c>
+      <x:c r="C16" s="2"/>
+      <x:c r="D16" s="2"/>
+      <x:c r="E16" s="2"/>
+      <x:c r="F16" s="2"/>
+      <x:c r="G16" s="2"/>
+      <x:c r="H16" s="2"/>
+      <x:c r="I16" s="2"/>
+      <x:c r="J16" s="2"/>
+      <x:c r="K16" s="2"/>
+      <x:c r="L16" s="2"/>
+      <x:c r="M16" s="2"/>
+      <x:c r="N16" s="2"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2"/>
+      <x:c r="B17" s="2"/>
+      <x:c r="C17" s="2"/>
+      <x:c r="D17" s="2"/>
+      <x:c r="E17" s="2"/>
+      <x:c r="F17" s="2"/>
+      <x:c r="G17" s="2"/>
+      <x:c r="H17" s="2"/>
+      <x:c r="I17" s="2"/>
+      <x:c r="J17" s="2"/>
+      <x:c r="K17" s="2"/>
+      <x:c r="L17" s="2"/>
+      <x:c r="M17" s="2"/>
+      <x:c r="N17" s="2"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2"/>
+      <x:c r="B18" s="2"/>
+      <x:c r="C18" s="2"/>
+      <x:c r="D18" s="2"/>
+      <x:c r="E18" s="2"/>
+      <x:c r="F18" s="2"/>
+      <x:c r="G18" s="2"/>
+      <x:c r="H18" s="2"/>
+      <x:c r="I18" s="2"/>
+      <x:c r="J18" s="2"/>
+      <x:c r="K18" s="2"/>
+      <x:c r="L18" s="2"/>
+      <x:c r="M18" s="2"/>
+      <x:c r="N18" s="2"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2"/>
+      <x:c r="B19" s="2"/>
+      <x:c r="C19" s="2"/>
+      <x:c r="D19" s="2"/>
+      <x:c r="E19" s="2"/>
+      <x:c r="F19" s="2"/>
+      <x:c r="G19" s="2"/>
+      <x:c r="H19" s="2"/>
+      <x:c r="I19" s="2"/>
+      <x:c r="J19" s="2"/>
+      <x:c r="K19" s="2"/>
+      <x:c r="L19" s="2"/>
+      <x:c r="M19" s="2"/>
+      <x:c r="N19" s="2"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2"/>
+      <x:c r="B20" s="2"/>
+      <x:c r="C20" s="2"/>
+      <x:c r="D20" s="2"/>
+      <x:c r="E20" s="2"/>
+      <x:c r="F20" s="2"/>
+      <x:c r="G20" s="2"/>
+      <x:c r="H20" s="2"/>
+      <x:c r="I20" s="2"/>
+      <x:c r="J20" s="2"/>
+      <x:c r="K20" s="2"/>
+      <x:c r="L20" s="2"/>
+      <x:c r="M20" s="2"/>
+      <x:c r="N20" s="2"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2"/>
+      <x:c r="B21" s="2"/>
+      <x:c r="C21" s="2"/>
+      <x:c r="D21" s="2"/>
+      <x:c r="E21" s="2"/>
+      <x:c r="F21" s="2"/>
+      <x:c r="G21" s="2"/>
+      <x:c r="H21" s="2"/>
+      <x:c r="I21" s="2"/>
+      <x:c r="J21" s="2"/>
+      <x:c r="K21" s="2"/>
+      <x:c r="L21" s="2"/>
+      <x:c r="M21" s="2"/>
+      <x:c r="N21" s="2"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2"/>
+      <x:c r="B22" s="2"/>
+      <x:c r="C22" s="2"/>
+      <x:c r="D22" s="2"/>
+      <x:c r="E22" s="2"/>
+      <x:c r="F22" s="2"/>
+      <x:c r="G22" s="2"/>
+      <x:c r="H22" s="2"/>
+      <x:c r="I22" s="2"/>
+      <x:c r="J22" s="2"/>
+      <x:c r="K22" s="2"/>
+      <x:c r="L22" s="2"/>
+      <x:c r="M22" s="2"/>
+      <x:c r="N22" s="2"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2"/>
+      <x:c r="B23" s="2"/>
+      <x:c r="C23" s="2"/>
+      <x:c r="D23" s="2"/>
+      <x:c r="E23" s="2"/>
+      <x:c r="F23" s="2"/>
+      <x:c r="G23" s="2"/>
+      <x:c r="H23" s="2"/>
+      <x:c r="I23" s="2"/>
+      <x:c r="J23" s="2"/>
+      <x:c r="K23" s="2"/>
+      <x:c r="L23" s="2"/>
+      <x:c r="M23" s="2"/>
+      <x:c r="N23" s="2"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2"/>
+      <x:c r="B24" s="2"/>
+      <x:c r="C24" s="2"/>
+      <x:c r="D24" s="2"/>
+      <x:c r="E24" s="2"/>
+      <x:c r="F24" s="2"/>
+      <x:c r="G24" s="2"/>
+      <x:c r="H24" s="2"/>
+      <x:c r="I24" s="2"/>
+      <x:c r="J24" s="2"/>
+      <x:c r="K24" s="2"/>
+      <x:c r="L24" s="2"/>
+      <x:c r="M24" s="2"/>
+      <x:c r="N24" s="2"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2"/>
+      <x:c r="B25" s="2"/>
+      <x:c r="C25" s="2"/>
+      <x:c r="D25" s="2"/>
+      <x:c r="E25" s="2"/>
+      <x:c r="F25" s="2"/>
+      <x:c r="G25" s="2"/>
+      <x:c r="H25" s="2"/>
+      <x:c r="I25" s="2"/>
+      <x:c r="J25" s="2"/>
+      <x:c r="K25" s="2"/>
+      <x:c r="L25" s="2"/>
+      <x:c r="M25" s="2"/>
+      <x:c r="N25" s="2"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2"/>
+      <x:c r="B26" s="2"/>
+      <x:c r="C26" s="2"/>
+      <x:c r="D26" s="2"/>
+      <x:c r="E26" s="2"/>
+      <x:c r="F26" s="2"/>
+      <x:c r="G26" s="2"/>
+      <x:c r="H26" s="2"/>
+      <x:c r="I26" s="2"/>
+      <x:c r="J26" s="2"/>
+      <x:c r="K26" s="2"/>
+      <x:c r="L26" s="2"/>
+      <x:c r="M26" s="2"/>
+      <x:c r="N26" s="2"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2"/>
+      <x:c r="B27" s="2"/>
+      <x:c r="C27" s="2"/>
+      <x:c r="D27" s="2"/>
+      <x:c r="E27" s="2"/>
+      <x:c r="F27" s="2"/>
+      <x:c r="G27" s="2"/>
+      <x:c r="H27" s="2"/>
+      <x:c r="I27" s="2"/>
+      <x:c r="J27" s="2"/>
+      <x:c r="K27" s="2"/>
+      <x:c r="L27" s="2"/>
+      <x:c r="M27" s="2"/>
+      <x:c r="N27" s="2"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2"/>
+      <x:c r="B28" s="2"/>
+      <x:c r="C28" s="2"/>
+      <x:c r="D28" s="2"/>
+      <x:c r="E28" s="2"/>
+      <x:c r="F28" s="2"/>
+      <x:c r="G28" s="2"/>
+      <x:c r="H28" s="2"/>
+      <x:c r="I28" s="2"/>
+      <x:c r="J28" s="2"/>
+      <x:c r="K28" s="2"/>
+      <x:c r="L28" s="2"/>
+      <x:c r="M28" s="2"/>
+      <x:c r="N28" s="2"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2"/>
+      <x:c r="B29" s="2"/>
+      <x:c r="C29" s="2"/>
+      <x:c r="D29" s="2"/>
+      <x:c r="E29" s="2"/>
+      <x:c r="F29" s="2"/>
+      <x:c r="G29" s="2"/>
+      <x:c r="H29" s="2"/>
+      <x:c r="I29" s="2"/>
+      <x:c r="J29" s="2"/>
+      <x:c r="K29" s="2"/>
+      <x:c r="L29" s="2"/>
+      <x:c r="M29" s="2"/>
+      <x:c r="N29" s="2"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2"/>
+      <x:c r="B30" s="2"/>
+      <x:c r="C30" s="2"/>
+      <x:c r="D30" s="2"/>
+      <x:c r="E30" s="2"/>
+      <x:c r="F30" s="2"/>
+      <x:c r="G30" s="2"/>
+      <x:c r="H30" s="2"/>
+      <x:c r="I30" s="2"/>
+      <x:c r="J30" s="2"/>
+      <x:c r="K30" s="2"/>
+      <x:c r="L30" s="2"/>
+      <x:c r="M30" s="2"/>
+      <x:c r="N30" s="2"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2"/>
+      <x:c r="B31" s="2"/>
+      <x:c r="C31" s="2"/>
+      <x:c r="D31" s="2"/>
+      <x:c r="E31" s="2"/>
+      <x:c r="F31" s="2"/>
+      <x:c r="G31" s="2"/>
+      <x:c r="H31" s="2"/>
+      <x:c r="I31" s="2"/>
+      <x:c r="J31" s="2"/>
+      <x:c r="K31" s="2"/>
+      <x:c r="L31" s="2"/>
+      <x:c r="M31" s="2"/>
+      <x:c r="N31" s="2"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2"/>
+      <x:c r="B32" s="2"/>
+      <x:c r="C32" s="2"/>
+      <x:c r="D32" s="2"/>
+      <x:c r="E32" s="2"/>
+      <x:c r="F32" s="2"/>
+      <x:c r="G32" s="2"/>
+      <x:c r="H32" s="2"/>
+      <x:c r="I32" s="2"/>
+      <x:c r="J32" s="2"/>
+      <x:c r="K32" s="2"/>
+      <x:c r="L32" s="2"/>
+      <x:c r="M32" s="2"/>
+      <x:c r="N32" s="2"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2"/>
+      <x:c r="B33" s="2"/>
+      <x:c r="C33" s="2"/>
+      <x:c r="D33" s="2"/>
+      <x:c r="E33" s="2"/>
+      <x:c r="F33" s="2"/>
+      <x:c r="G33" s="2"/>
+      <x:c r="H33" s="2"/>
+      <x:c r="I33" s="2"/>
+      <x:c r="J33" s="2"/>
+      <x:c r="K33" s="2"/>
+      <x:c r="L33" s="2"/>
+      <x:c r="M33" s="2"/>
+      <x:c r="N33" s="2"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2"/>
+      <x:c r="B34" s="2"/>
+      <x:c r="C34" s="2"/>
+      <x:c r="D34" s="2"/>
+      <x:c r="E34" s="2"/>
+      <x:c r="F34" s="2"/>
+      <x:c r="G34" s="2"/>
+      <x:c r="H34" s="2"/>
+      <x:c r="I34" s="2"/>
+      <x:c r="J34" s="2"/>
+      <x:c r="K34" s="2"/>
+      <x:c r="L34" s="2"/>
+      <x:c r="M34" s="2"/>
+      <x:c r="N34" s="2"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2"/>
+      <x:c r="B35" s="2"/>
+      <x:c r="C35" s="2"/>
+      <x:c r="D35" s="2"/>
+      <x:c r="E35" s="2"/>
+      <x:c r="F35" s="2"/>
+      <x:c r="G35" s="2"/>
+      <x:c r="H35" s="2"/>
+      <x:c r="I35" s="2"/>
+      <x:c r="J35" s="2"/>
+      <x:c r="K35" s="2"/>
+      <x:c r="L35" s="2"/>
+      <x:c r="M35" s="2"/>
+      <x:c r="N35" s="2"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2"/>
+      <x:c r="B36" s="2"/>
+      <x:c r="C36" s="2"/>
+      <x:c r="D36" s="2"/>
+      <x:c r="E36" s="2"/>
+      <x:c r="F36" s="2"/>
+      <x:c r="G36" s="2"/>
+      <x:c r="H36" s="2"/>
+      <x:c r="I36" s="2"/>
+      <x:c r="J36" s="2"/>
+      <x:c r="K36" s="2"/>
+      <x:c r="L36" s="2"/>
+      <x:c r="M36" s="2"/>
+      <x:c r="N36" s="2"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2"/>
+      <x:c r="B37" s="2"/>
+      <x:c r="C37" s="2"/>
+      <x:c r="D37" s="2"/>
+      <x:c r="E37" s="2"/>
+      <x:c r="F37" s="2"/>
+      <x:c r="G37" s="2"/>
+      <x:c r="H37" s="2"/>
+      <x:c r="I37" s="2"/>
+      <x:c r="J37" s="2"/>
+      <x:c r="K37" s="2"/>
+      <x:c r="L37" s="2"/>
+      <x:c r="M37" s="2"/>
+      <x:c r="N37" s="2"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2"/>
+      <x:c r="B38" s="2"/>
+      <x:c r="C38" s="2"/>
+      <x:c r="D38" s="2"/>
+      <x:c r="E38" s="2"/>
+      <x:c r="F38" s="2"/>
+      <x:c r="G38" s="2"/>
+      <x:c r="H38" s="2"/>
+      <x:c r="I38" s="2"/>
+      <x:c r="J38" s="2"/>
+      <x:c r="K38" s="2"/>
+      <x:c r="L38" s="2"/>
+      <x:c r="M38" s="2"/>
+      <x:c r="N38" s="2"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2"/>
+      <x:c r="B39" s="2"/>
+      <x:c r="C39" s="2"/>
+      <x:c r="D39" s="2"/>
+      <x:c r="E39" s="2"/>
+      <x:c r="F39" s="2"/>
+      <x:c r="G39" s="2"/>
+      <x:c r="H39" s="2"/>
+      <x:c r="I39" s="2"/>
+      <x:c r="J39" s="2"/>
+      <x:c r="K39" s="2"/>
+      <x:c r="L39" s="2"/>
+      <x:c r="M39" s="2"/>
+      <x:c r="N39" s="2"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2"/>
+      <x:c r="B40" s="2"/>
+      <x:c r="C40" s="2"/>
+      <x:c r="D40" s="2"/>
+      <x:c r="E40" s="2"/>
+      <x:c r="F40" s="2"/>
+      <x:c r="G40" s="2"/>
+      <x:c r="H40" s="2"/>
+      <x:c r="I40" s="2"/>
+      <x:c r="J40" s="2"/>
+      <x:c r="K40" s="2"/>
+      <x:c r="L40" s="2"/>
+      <x:c r="M40" s="2"/>
+      <x:c r="N40" s="2"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="2"/>
+      <x:c r="B41" s="2"/>
+      <x:c r="C41" s="2"/>
+      <x:c r="D41" s="2"/>
+      <x:c r="E41" s="2"/>
+      <x:c r="F41" s="2"/>
+      <x:c r="G41" s="2"/>
+      <x:c r="H41" s="2"/>
+      <x:c r="I41" s="2"/>
+      <x:c r="J41" s="2"/>
+      <x:c r="K41" s="2"/>
+      <x:c r="L41" s="2"/>
+      <x:c r="M41" s="2"/>
+      <x:c r="N41" s="2"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2"/>
+      <x:c r="B42" s="2"/>
+      <x:c r="C42" s="2"/>
+      <x:c r="D42" s="2"/>
+      <x:c r="E42" s="2"/>
+      <x:c r="F42" s="2"/>
+      <x:c r="G42" s="2"/>
+      <x:c r="H42" s="2"/>
+      <x:c r="I42" s="2"/>
+      <x:c r="J42" s="2"/>
+      <x:c r="K42" s="2"/>
+      <x:c r="L42" s="2"/>
+      <x:c r="M42" s="2"/>
+      <x:c r="N42" s="2"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2"/>
+      <x:c r="B43" s="2"/>
+      <x:c r="C43" s="2"/>
+      <x:c r="D43" s="2"/>
+      <x:c r="E43" s="2"/>
+      <x:c r="F43" s="2"/>
+      <x:c r="G43" s="2"/>
+      <x:c r="H43" s="2"/>
+      <x:c r="I43" s="2"/>
+      <x:c r="J43" s="2"/>
+      <x:c r="K43" s="2"/>
+      <x:c r="L43" s="2"/>
+      <x:c r="M43" s="2"/>
+      <x:c r="N43" s="2"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2"/>
+      <x:c r="B44" s="2"/>
+      <x:c r="C44" s="2"/>
+      <x:c r="D44" s="2"/>
+      <x:c r="E44" s="2"/>
+      <x:c r="F44" s="2"/>
+      <x:c r="G44" s="2"/>
+      <x:c r="H44" s="2"/>
+      <x:c r="I44" s="2"/>
+      <x:c r="J44" s="2"/>
+      <x:c r="K44" s="2"/>
+      <x:c r="L44" s="2"/>
+      <x:c r="M44" s="2"/>
+      <x:c r="N44" s="2"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2"/>
+      <x:c r="B45" s="2"/>
+      <x:c r="C45" s="2"/>
+      <x:c r="D45" s="2"/>
+      <x:c r="E45" s="2"/>
+      <x:c r="F45" s="2"/>
+      <x:c r="G45" s="2"/>
+      <x:c r="H45" s="2"/>
+      <x:c r="I45" s="2"/>
+      <x:c r="J45" s="2"/>
+      <x:c r="K45" s="2"/>
+      <x:c r="L45" s="2"/>
+      <x:c r="M45" s="2"/>
+      <x:c r="N45" s="2"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2"/>
+      <x:c r="B46" s="2"/>
+      <x:c r="C46" s="2"/>
+      <x:c r="D46" s="2"/>
+      <x:c r="E46" s="2"/>
+      <x:c r="F46" s="2"/>
+      <x:c r="G46" s="2"/>
+      <x:c r="H46" s="2"/>
+      <x:c r="I46" s="2"/>
+      <x:c r="J46" s="2"/>
+      <x:c r="K46" s="2"/>
+      <x:c r="L46" s="2"/>
+      <x:c r="M46" s="2"/>
+      <x:c r="N46" s="2"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2"/>
+      <x:c r="B47" s="2"/>
+      <x:c r="C47" s="2"/>
+      <x:c r="D47" s="2"/>
+      <x:c r="E47" s="2"/>
+      <x:c r="F47" s="2"/>
+      <x:c r="G47" s="2"/>
+      <x:c r="H47" s="2"/>
+      <x:c r="I47" s="2"/>
+      <x:c r="J47" s="2"/>
+      <x:c r="K47" s="2"/>
+      <x:c r="L47" s="2"/>
+      <x:c r="M47" s="2"/>
+      <x:c r="N47" s="2"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2"/>
+      <x:c r="B48" s="2"/>
+      <x:c r="C48" s="2"/>
+      <x:c r="D48" s="2"/>
+      <x:c r="E48" s="2"/>
+      <x:c r="F48" s="2"/>
+      <x:c r="G48" s="2"/>
+      <x:c r="H48" s="2"/>
+      <x:c r="I48" s="2"/>
+      <x:c r="J48" s="2"/>
+      <x:c r="K48" s="2"/>
+      <x:c r="L48" s="2"/>
+      <x:c r="M48" s="2"/>
+      <x:c r="N48" s="2"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2"/>
+      <x:c r="B49" s="2"/>
+      <x:c r="C49" s="2"/>
+      <x:c r="D49" s="2"/>
+      <x:c r="E49" s="2"/>
+      <x:c r="F49" s="2"/>
+      <x:c r="G49" s="2"/>
+      <x:c r="H49" s="2"/>
+      <x:c r="I49" s="2"/>
+      <x:c r="J49" s="2"/>
+      <x:c r="K49" s="2"/>
+      <x:c r="L49" s="2"/>
+      <x:c r="M49" s="2"/>
+      <x:c r="N49" s="2"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2"/>
+      <x:c r="B50" s="2"/>
+      <x:c r="C50" s="2"/>
+      <x:c r="D50" s="2"/>
+      <x:c r="E50" s="2"/>
+      <x:c r="F50" s="2"/>
+      <x:c r="G50" s="2"/>
+      <x:c r="H50" s="2"/>
+      <x:c r="I50" s="2"/>
+      <x:c r="J50" s="2"/>
+      <x:c r="K50" s="2"/>
+      <x:c r="L50" s="2"/>
+      <x:c r="M50" s="2"/>
+      <x:c r="N50" s="2"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2"/>
+      <x:c r="B51" s="2"/>
+      <x:c r="C51" s="2"/>
+      <x:c r="D51" s="2"/>
+      <x:c r="E51" s="2"/>
+      <x:c r="F51" s="2"/>
+      <x:c r="G51" s="2"/>
+      <x:c r="H51" s="2"/>
+      <x:c r="I51" s="2"/>
+      <x:c r="J51" s="2"/>
+      <x:c r="K51" s="2"/>
+      <x:c r="L51" s="2"/>
+      <x:c r="M51" s="2"/>
+      <x:c r="N51" s="2"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2"/>
+      <x:c r="B52" s="2"/>
+      <x:c r="C52" s="2"/>
+      <x:c r="D52" s="2"/>
+      <x:c r="E52" s="2"/>
+      <x:c r="F52" s="2"/>
+      <x:c r="G52" s="2"/>
+      <x:c r="H52" s="2"/>
+      <x:c r="I52" s="2"/>
+      <x:c r="J52" s="2"/>
+      <x:c r="K52" s="2"/>
+      <x:c r="L52" s="2"/>
+      <x:c r="M52" s="2"/>
+      <x:c r="N52" s="2"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="2"/>
+      <x:c r="B53" s="2"/>
+      <x:c r="C53" s="2"/>
+      <x:c r="D53" s="2"/>
+      <x:c r="E53" s="2"/>
+      <x:c r="F53" s="2"/>
+      <x:c r="G53" s="2"/>
+      <x:c r="H53" s="2"/>
+      <x:c r="I53" s="2"/>
+      <x:c r="J53" s="2"/>
+      <x:c r="K53" s="2"/>
+      <x:c r="L53" s="2"/>
+      <x:c r="M53" s="2"/>
+      <x:c r="N53" s="2"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="2"/>
+      <x:c r="B54" s="2"/>
+      <x:c r="C54" s="2"/>
+      <x:c r="D54" s="2"/>
+      <x:c r="E54" s="2"/>
+      <x:c r="F54" s="2"/>
+      <x:c r="G54" s="2"/>
+      <x:c r="H54" s="2"/>
+      <x:c r="I54" s="2"/>
+      <x:c r="J54" s="2"/>
+      <x:c r="K54" s="2"/>
+      <x:c r="L54" s="2"/>
+      <x:c r="M54" s="2"/>
+      <x:c r="N54" s="2"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2"/>
+      <x:c r="B55" s="2"/>
+      <x:c r="C55" s="2"/>
+      <x:c r="D55" s="2"/>
+      <x:c r="E55" s="2"/>
+      <x:c r="F55" s="2"/>
+      <x:c r="G55" s="2"/>
+      <x:c r="H55" s="2"/>
+      <x:c r="I55" s="2"/>
+      <x:c r="J55" s="2"/>
+      <x:c r="K55" s="2"/>
+      <x:c r="L55" s="2"/>
+      <x:c r="M55" s="2"/>
+      <x:c r="N55" s="2"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2"/>
+      <x:c r="B56" s="2"/>
+      <x:c r="C56" s="2"/>
+      <x:c r="D56" s="2"/>
+      <x:c r="E56" s="2"/>
+      <x:c r="F56" s="2"/>
+      <x:c r="G56" s="2"/>
+      <x:c r="H56" s="2"/>
+      <x:c r="I56" s="2"/>
+      <x:c r="J56" s="2"/>
+      <x:c r="K56" s="2"/>
+      <x:c r="L56" s="2"/>
+      <x:c r="M56" s="2"/>
+      <x:c r="N56" s="2"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2"/>
+      <x:c r="B57" s="2"/>
+      <x:c r="C57" s="2"/>
+      <x:c r="D57" s="2"/>
+      <x:c r="E57" s="2"/>
+      <x:c r="F57" s="2"/>
+      <x:c r="G57" s="2"/>
+      <x:c r="H57" s="2"/>
+      <x:c r="I57" s="2"/>
+      <x:c r="J57" s="2"/>
+      <x:c r="K57" s="2"/>
+      <x:c r="L57" s="2"/>
+      <x:c r="M57" s="2"/>
+      <x:c r="N57" s="2"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2"/>
+      <x:c r="B58" s="2"/>
+      <x:c r="C58" s="2"/>
+      <x:c r="D58" s="2"/>
+      <x:c r="E58" s="2"/>
+      <x:c r="F58" s="2"/>
+      <x:c r="G58" s="2"/>
+      <x:c r="H58" s="2"/>
+      <x:c r="I58" s="2"/>
+      <x:c r="J58" s="2"/>
+      <x:c r="K58" s="2"/>
+      <x:c r="L58" s="2"/>
+      <x:c r="M58" s="2"/>
+      <x:c r="N58" s="2"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2"/>
+      <x:c r="B59" s="2"/>
+      <x:c r="C59" s="2"/>
+      <x:c r="D59" s="2"/>
+      <x:c r="E59" s="2"/>
+      <x:c r="F59" s="2"/>
+      <x:c r="G59" s="2"/>
+      <x:c r="H59" s="2"/>
+      <x:c r="I59" s="2"/>
+      <x:c r="J59" s="2"/>
+      <x:c r="K59" s="2"/>
+      <x:c r="L59" s="2"/>
+      <x:c r="M59" s="2"/>
+      <x:c r="N59" s="2"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2"/>
+      <x:c r="B60" s="2"/>
+      <x:c r="C60" s="2"/>
+      <x:c r="D60" s="2"/>
+      <x:c r="E60" s="2"/>
+      <x:c r="F60" s="2"/>
+      <x:c r="G60" s="2"/>
+      <x:c r="H60" s="2"/>
+      <x:c r="I60" s="2"/>
+      <x:c r="J60" s="2"/>
+      <x:c r="K60" s="2"/>
+      <x:c r="L60" s="2"/>
+      <x:c r="M60" s="2"/>
+      <x:c r="N60" s="2"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="2"/>
+      <x:c r="B61" s="2"/>
+      <x:c r="C61" s="2"/>
+      <x:c r="D61" s="2"/>
+      <x:c r="E61" s="2"/>
+      <x:c r="F61" s="2"/>
+      <x:c r="G61" s="2"/>
+      <x:c r="H61" s="2"/>
+      <x:c r="I61" s="2"/>
+      <x:c r="J61" s="2"/>
+      <x:c r="K61" s="2"/>
+      <x:c r="L61" s="2"/>
+      <x:c r="M61" s="2"/>
+      <x:c r="N61" s="2"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2"/>
+      <x:c r="B62" s="2"/>
+      <x:c r="C62" s="2"/>
+      <x:c r="D62" s="2"/>
+      <x:c r="E62" s="2"/>
+      <x:c r="F62" s="2"/>
+      <x:c r="G62" s="2"/>
+      <x:c r="H62" s="2"/>
+      <x:c r="I62" s="2"/>
+      <x:c r="J62" s="2"/>
+      <x:c r="K62" s="2"/>
+      <x:c r="L62" s="2"/>
+      <x:c r="M62" s="2"/>
+      <x:c r="N62" s="2"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="2"/>
+      <x:c r="B63" s="2"/>
+      <x:c r="C63" s="2"/>
+      <x:c r="D63" s="2"/>
+      <x:c r="E63" s="2"/>
+      <x:c r="F63" s="2"/>
+      <x:c r="G63" s="2"/>
+      <x:c r="H63" s="2"/>
+      <x:c r="I63" s="2"/>
+      <x:c r="J63" s="2"/>
+      <x:c r="K63" s="2"/>
+      <x:c r="L63" s="2"/>
+      <x:c r="M63" s="2"/>
+      <x:c r="N63" s="2"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="2"/>
+      <x:c r="B64" s="2"/>
+      <x:c r="C64" s="2"/>
+      <x:c r="D64" s="2"/>
+      <x:c r="E64" s="2"/>
+      <x:c r="F64" s="2"/>
+      <x:c r="G64" s="2"/>
+      <x:c r="H64" s="2"/>
+      <x:c r="I64" s="2"/>
+      <x:c r="J64" s="2"/>
+      <x:c r="K64" s="2"/>
+      <x:c r="L64" s="2"/>
+      <x:c r="M64" s="2"/>
+      <x:c r="N64" s="2"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="2"/>
+      <x:c r="B65" s="2"/>
+      <x:c r="C65" s="2"/>
+      <x:c r="D65" s="2"/>
+      <x:c r="E65" s="2"/>
+      <x:c r="F65" s="2"/>
+      <x:c r="G65" s="2"/>
+      <x:c r="H65" s="2"/>
+      <x:c r="I65" s="2"/>
+      <x:c r="J65" s="2"/>
+      <x:c r="K65" s="2"/>
+      <x:c r="L65" s="2"/>
+      <x:c r="M65" s="2"/>
+      <x:c r="N65" s="2"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="2"/>
+      <x:c r="B66" s="2"/>
+      <x:c r="C66" s="2"/>
+      <x:c r="D66" s="2"/>
+      <x:c r="E66" s="2"/>
+      <x:c r="F66" s="2"/>
+      <x:c r="G66" s="2"/>
+      <x:c r="H66" s="2"/>
+      <x:c r="I66" s="2"/>
+      <x:c r="J66" s="2"/>
+      <x:c r="K66" s="2"/>
+      <x:c r="L66" s="2"/>
+      <x:c r="M66" s="2"/>
+      <x:c r="N66" s="2"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="2"/>
+      <x:c r="B67" s="2"/>
+      <x:c r="C67" s="2"/>
+      <x:c r="D67" s="2"/>
+      <x:c r="E67" s="2"/>
+      <x:c r="F67" s="2"/>
+      <x:c r="G67" s="2"/>
+      <x:c r="H67" s="2"/>
+      <x:c r="I67" s="2"/>
+      <x:c r="J67" s="2"/>
+      <x:c r="K67" s="2"/>
+      <x:c r="L67" s="2"/>
+      <x:c r="M67" s="2"/>
+      <x:c r="N67" s="2"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="2"/>
+      <x:c r="B68" s="2"/>
+      <x:c r="C68" s="2"/>
+      <x:c r="D68" s="2"/>
+      <x:c r="E68" s="2"/>
+      <x:c r="F68" s="2"/>
+      <x:c r="G68" s="2"/>
+      <x:c r="H68" s="2"/>
+      <x:c r="I68" s="2"/>
+      <x:c r="J68" s="2"/>
+      <x:c r="K68" s="2"/>
+      <x:c r="L68" s="2"/>
+      <x:c r="M68" s="2"/>
+      <x:c r="N68" s="2"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="2"/>
+      <x:c r="B69" s="2"/>
+      <x:c r="C69" s="2"/>
+      <x:c r="D69" s="2"/>
+      <x:c r="E69" s="2"/>
+      <x:c r="F69" s="2"/>
+      <x:c r="G69" s="2"/>
+      <x:c r="H69" s="2"/>
+      <x:c r="I69" s="2"/>
+      <x:c r="J69" s="2"/>
+      <x:c r="K69" s="2"/>
+      <x:c r="L69" s="2"/>
+      <x:c r="M69" s="2"/>
+      <x:c r="N69" s="2"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="2"/>
+      <x:c r="B70" s="2"/>
+      <x:c r="C70" s="2"/>
+      <x:c r="D70" s="2"/>
+      <x:c r="E70" s="2"/>
+      <x:c r="F70" s="2"/>
+      <x:c r="G70" s="2"/>
+      <x:c r="H70" s="2"/>
+      <x:c r="I70" s="2"/>
+      <x:c r="J70" s="2"/>
+      <x:c r="K70" s="2"/>
+      <x:c r="L70" s="2"/>
+      <x:c r="M70" s="2"/>
+      <x:c r="N70" s="2"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="2"/>
+      <x:c r="B71" s="2"/>
+      <x:c r="C71" s="2"/>
+      <x:c r="D71" s="2"/>
+      <x:c r="E71" s="2"/>
+      <x:c r="F71" s="2"/>
+      <x:c r="G71" s="2"/>
+      <x:c r="H71" s="2"/>
+      <x:c r="I71" s="2"/>
+      <x:c r="J71" s="2"/>
+      <x:c r="K71" s="2"/>
+      <x:c r="L71" s="2"/>
+      <x:c r="M71" s="2"/>
+      <x:c r="N71" s="2"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="2"/>
+      <x:c r="B72" s="2"/>
+      <x:c r="C72" s="2"/>
+      <x:c r="D72" s="2"/>
+      <x:c r="E72" s="2"/>
+      <x:c r="F72" s="2"/>
+      <x:c r="G72" s="2"/>
+      <x:c r="H72" s="2"/>
+      <x:c r="I72" s="2"/>
+      <x:c r="J72" s="2"/>
+      <x:c r="K72" s="2"/>
+      <x:c r="L72" s="2"/>
+      <x:c r="M72" s="2"/>
+      <x:c r="N72" s="2"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="2"/>
+      <x:c r="B73" s="2"/>
+      <x:c r="C73" s="2"/>
+      <x:c r="D73" s="2"/>
+      <x:c r="E73" s="2"/>
+      <x:c r="F73" s="2"/>
+      <x:c r="G73" s="2"/>
+      <x:c r="H73" s="2"/>
+      <x:c r="I73" s="2"/>
+      <x:c r="J73" s="2"/>
+      <x:c r="K73" s="2"/>
+      <x:c r="L73" s="2"/>
+      <x:c r="M73" s="2"/>
+      <x:c r="N73" s="2"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="2"/>
+      <x:c r="B74" s="2"/>
+      <x:c r="C74" s="2"/>
+      <x:c r="D74" s="2"/>
+      <x:c r="E74" s="2"/>
+      <x:c r="F74" s="2"/>
+      <x:c r="G74" s="2"/>
+      <x:c r="H74" s="2"/>
+      <x:c r="I74" s="2"/>
+      <x:c r="J74" s="2"/>
+      <x:c r="K74" s="2"/>
+      <x:c r="L74" s="2"/>
+      <x:c r="M74" s="2"/>
+      <x:c r="N74" s="2"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="2"/>
+      <x:c r="B75" s="2"/>
+      <x:c r="C75" s="2"/>
+      <x:c r="D75" s="2"/>
+      <x:c r="E75" s="2"/>
+      <x:c r="F75" s="2"/>
+      <x:c r="G75" s="2"/>
+      <x:c r="H75" s="2"/>
+      <x:c r="I75" s="2"/>
+      <x:c r="J75" s="2"/>
+      <x:c r="K75" s="2"/>
+      <x:c r="L75" s="2"/>
+      <x:c r="M75" s="2"/>
+      <x:c r="N75" s="2"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="2"/>
+      <x:c r="B76" s="2"/>
+      <x:c r="C76" s="2"/>
+      <x:c r="D76" s="2"/>
+      <x:c r="E76" s="2"/>
+      <x:c r="F76" s="2"/>
+      <x:c r="G76" s="2"/>
+      <x:c r="H76" s="2"/>
+      <x:c r="I76" s="2"/>
+      <x:c r="J76" s="2"/>
+      <x:c r="K76" s="2"/>
+      <x:c r="L76" s="2"/>
+      <x:c r="M76" s="2"/>
+      <x:c r="N76" s="2"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="2"/>
+      <x:c r="B77" s="2"/>
+      <x:c r="C77" s="2"/>
+      <x:c r="D77" s="2"/>
+      <x:c r="E77" s="2"/>
+      <x:c r="F77" s="2"/>
+      <x:c r="G77" s="2"/>
+      <x:c r="H77" s="2"/>
+      <x:c r="I77" s="2"/>
+      <x:c r="J77" s="2"/>
+      <x:c r="K77" s="2"/>
+      <x:c r="L77" s="2"/>
+      <x:c r="M77" s="2"/>
+      <x:c r="N77" s="2"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="2"/>
+      <x:c r="B78" s="2"/>
+      <x:c r="C78" s="2"/>
+      <x:c r="D78" s="2"/>
+      <x:c r="E78" s="2"/>
+      <x:c r="F78" s="2"/>
+      <x:c r="G78" s="2"/>
+      <x:c r="H78" s="2"/>
+      <x:c r="I78" s="2"/>
+      <x:c r="J78" s="2"/>
+      <x:c r="K78" s="2"/>
+      <x:c r="L78" s="2"/>
+      <x:c r="M78" s="2"/>
+      <x:c r="N78" s="2"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="2"/>
+      <x:c r="B79" s="2"/>
+      <x:c r="C79" s="2"/>
+      <x:c r="D79" s="2"/>
+      <x:c r="E79" s="2"/>
+      <x:c r="F79" s="2"/>
+      <x:c r="G79" s="2"/>
+      <x:c r="H79" s="2"/>
+      <x:c r="I79" s="2"/>
+      <x:c r="J79" s="2"/>
+      <x:c r="K79" s="2"/>
+      <x:c r="L79" s="2"/>
+      <x:c r="M79" s="2"/>
+      <x:c r="N79" s="2"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="2"/>
+      <x:c r="B80" s="2"/>
+      <x:c r="C80" s="2"/>
+      <x:c r="D80" s="2"/>
+      <x:c r="E80" s="2"/>
+      <x:c r="F80" s="2"/>
+      <x:c r="G80" s="2"/>
+      <x:c r="H80" s="2"/>
+      <x:c r="I80" s="2"/>
+      <x:c r="J80" s="2"/>
+      <x:c r="K80" s="2"/>
+      <x:c r="L80" s="2"/>
+      <x:c r="M80" s="2"/>
+      <x:c r="N80" s="2"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="2"/>
+      <x:c r="B81" s="2"/>
+      <x:c r="C81" s="2"/>
+      <x:c r="D81" s="2"/>
+      <x:c r="E81" s="2"/>
+      <x:c r="F81" s="2"/>
+      <x:c r="G81" s="2"/>
+      <x:c r="H81" s="2"/>
+      <x:c r="I81" s="2"/>
+      <x:c r="J81" s="2"/>
+      <x:c r="K81" s="2"/>
+      <x:c r="L81" s="2"/>
+      <x:c r="M81" s="2"/>
+      <x:c r="N81" s="2"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="2"/>
+      <x:c r="B82" s="2"/>
+      <x:c r="C82" s="2"/>
+      <x:c r="D82" s="2"/>
+      <x:c r="E82" s="2"/>
+      <x:c r="F82" s="2"/>
+      <x:c r="G82" s="2"/>
+      <x:c r="H82" s="2"/>
+      <x:c r="I82" s="2"/>
+      <x:c r="J82" s="2"/>
+      <x:c r="K82" s="2"/>
+      <x:c r="L82" s="2"/>
+      <x:c r="M82" s="2"/>
+      <x:c r="N82" s="2"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="2"/>
+      <x:c r="B83" s="2"/>
+      <x:c r="C83" s="2"/>
+      <x:c r="D83" s="2"/>
+      <x:c r="E83" s="2"/>
+      <x:c r="F83" s="2"/>
+      <x:c r="G83" s="2"/>
+      <x:c r="H83" s="2"/>
+      <x:c r="I83" s="2"/>
+      <x:c r="J83" s="2"/>
+      <x:c r="K83" s="2"/>
+      <x:c r="L83" s="2"/>
+      <x:c r="M83" s="2"/>
+      <x:c r="N83" s="2"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="2"/>
+      <x:c r="B84" s="2"/>
+      <x:c r="C84" s="2"/>
+      <x:c r="D84" s="2"/>
+      <x:c r="E84" s="2"/>
+      <x:c r="F84" s="2"/>
+      <x:c r="G84" s="2"/>
+      <x:c r="H84" s="2"/>
+      <x:c r="I84" s="2"/>
+      <x:c r="J84" s="2"/>
+      <x:c r="K84" s="2"/>
+      <x:c r="L84" s="2"/>
+      <x:c r="M84" s="2"/>
+      <x:c r="N84" s="2"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="2"/>
+      <x:c r="B85" s="2"/>
+      <x:c r="C85" s="2"/>
+      <x:c r="D85" s="2"/>
+      <x:c r="E85" s="2"/>
+      <x:c r="F85" s="2"/>
+      <x:c r="G85" s="2"/>
+      <x:c r="H85" s="2"/>
+      <x:c r="I85" s="2"/>
+      <x:c r="J85" s="2"/>
+      <x:c r="K85" s="2"/>
+      <x:c r="L85" s="2"/>
+      <x:c r="M85" s="2"/>
+      <x:c r="N85" s="2"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="2"/>
+      <x:c r="B86" s="2"/>
+      <x:c r="C86" s="2"/>
+      <x:c r="D86" s="2"/>
+      <x:c r="E86" s="2"/>
+      <x:c r="F86" s="2"/>
+      <x:c r="G86" s="2"/>
+      <x:c r="H86" s="2"/>
+      <x:c r="I86" s="2"/>
+      <x:c r="J86" s="2"/>
+      <x:c r="K86" s="2"/>
+      <x:c r="L86" s="2"/>
+      <x:c r="M86" s="2"/>
+      <x:c r="N86" s="2"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="2"/>
+      <x:c r="B87" s="2"/>
+      <x:c r="C87" s="2"/>
+      <x:c r="D87" s="2"/>
+      <x:c r="E87" s="2"/>
+      <x:c r="F87" s="2"/>
+      <x:c r="G87" s="2"/>
+      <x:c r="H87" s="2"/>
+      <x:c r="I87" s="2"/>
+      <x:c r="J87" s="2"/>
+      <x:c r="K87" s="2"/>
+      <x:c r="L87" s="2"/>
+      <x:c r="M87" s="2"/>
+      <x:c r="N87" s="2"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="2"/>
+      <x:c r="B88" s="2"/>
+      <x:c r="C88" s="2"/>
+      <x:c r="D88" s="2"/>
+      <x:c r="E88" s="2"/>
+      <x:c r="F88" s="2"/>
+      <x:c r="G88" s="2"/>
+      <x:c r="H88" s="2"/>
+      <x:c r="I88" s="2"/>
+      <x:c r="J88" s="2"/>
+      <x:c r="K88" s="2"/>
+      <x:c r="L88" s="2"/>
+      <x:c r="M88" s="2"/>
+      <x:c r="N88" s="2"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="2"/>
+      <x:c r="B89" s="2"/>
+      <x:c r="C89" s="2"/>
+      <x:c r="D89" s="2"/>
+      <x:c r="E89" s="2"/>
+      <x:c r="F89" s="2"/>
+      <x:c r="G89" s="2"/>
+      <x:c r="H89" s="2"/>
+      <x:c r="I89" s="2"/>
+      <x:c r="J89" s="2"/>
+      <x:c r="K89" s="2"/>
+      <x:c r="L89" s="2"/>
+      <x:c r="M89" s="2"/>
+      <x:c r="N89" s="2"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="2"/>
+      <x:c r="B90" s="2"/>
+      <x:c r="C90" s="2"/>
+      <x:c r="D90" s="2"/>
+      <x:c r="E90" s="2"/>
+      <x:c r="F90" s="2"/>
+      <x:c r="G90" s="2"/>
+      <x:c r="H90" s="2"/>
+      <x:c r="I90" s="2"/>
+      <x:c r="J90" s="2"/>
+      <x:c r="K90" s="2"/>
+      <x:c r="L90" s="2"/>
+      <x:c r="M90" s="2"/>
+      <x:c r="N90" s="2"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="2"/>
+      <x:c r="B91" s="2"/>
+      <x:c r="C91" s="2"/>
+      <x:c r="D91" s="2"/>
+      <x:c r="E91" s="2"/>
+      <x:c r="F91" s="2"/>
+      <x:c r="G91" s="2"/>
+      <x:c r="H91" s="2"/>
+      <x:c r="I91" s="2"/>
+      <x:c r="J91" s="2"/>
+      <x:c r="K91" s="2"/>
+      <x:c r="L91" s="2"/>
+      <x:c r="M91" s="2"/>
+      <x:c r="N91" s="2"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="2"/>
+      <x:c r="B92" s="2"/>
+      <x:c r="C92" s="2"/>
+      <x:c r="D92" s="2"/>
+      <x:c r="E92" s="2"/>
+      <x:c r="F92" s="2"/>
+      <x:c r="G92" s="2"/>
+      <x:c r="H92" s="2"/>
+      <x:c r="I92" s="2"/>
+      <x:c r="J92" s="2"/>
+      <x:c r="K92" s="2"/>
+      <x:c r="L92" s="2"/>
+      <x:c r="M92" s="2"/>
+      <x:c r="N92" s="2"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="2"/>
+      <x:c r="B93" s="2"/>
+      <x:c r="C93" s="2"/>
+      <x:c r="D93" s="2"/>
+      <x:c r="E93" s="2"/>
+      <x:c r="F93" s="2"/>
+      <x:c r="G93" s="2"/>
+      <x:c r="H93" s="2"/>
+      <x:c r="I93" s="2"/>
+      <x:c r="J93" s="2"/>
+      <x:c r="K93" s="2"/>
+      <x:c r="L93" s="2"/>
+      <x:c r="M93" s="2"/>
+      <x:c r="N93" s="2"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="2"/>
+      <x:c r="B94" s="2"/>
+      <x:c r="C94" s="2"/>
+      <x:c r="D94" s="2"/>
+      <x:c r="E94" s="2"/>
+      <x:c r="F94" s="2"/>
+      <x:c r="G94" s="2"/>
+      <x:c r="H94" s="2"/>
+      <x:c r="I94" s="2"/>
+      <x:c r="J94" s="2"/>
+      <x:c r="K94" s="2"/>
+      <x:c r="L94" s="2"/>
+      <x:c r="M94" s="2"/>
+      <x:c r="N94" s="2"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="2"/>
+      <x:c r="B95" s="2"/>
+      <x:c r="C95" s="2"/>
+      <x:c r="D95" s="2"/>
+      <x:c r="E95" s="2"/>
+      <x:c r="F95" s="2"/>
+      <x:c r="G95" s="2"/>
+      <x:c r="H95" s="2"/>
+      <x:c r="I95" s="2"/>
+      <x:c r="J95" s="2"/>
+      <x:c r="K95" s="2"/>
+      <x:c r="L95" s="2"/>
+      <x:c r="M95" s="2"/>
+      <x:c r="N95" s="2"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="2"/>
+      <x:c r="B96" s="2"/>
+      <x:c r="C96" s="2"/>
+      <x:c r="D96" s="2"/>
+      <x:c r="E96" s="2"/>
+      <x:c r="F96" s="2"/>
+      <x:c r="G96" s="2"/>
+      <x:c r="H96" s="2"/>
+      <x:c r="I96" s="2"/>
+      <x:c r="J96" s="2"/>
+      <x:c r="K96" s="2"/>
+      <x:c r="L96" s="2"/>
+      <x:c r="M96" s="2"/>
+      <x:c r="N96" s="2"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="2"/>
+      <x:c r="B97" s="2"/>
+      <x:c r="C97" s="2"/>
+      <x:c r="D97" s="2"/>
+      <x:c r="E97" s="2"/>
+      <x:c r="F97" s="2"/>
+      <x:c r="G97" s="2"/>
+      <x:c r="H97" s="2"/>
+      <x:c r="I97" s="2"/>
+      <x:c r="J97" s="2"/>
+      <x:c r="K97" s="2"/>
+      <x:c r="L97" s="2"/>
+      <x:c r="M97" s="2"/>
+      <x:c r="N97" s="2"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="2"/>
+      <x:c r="B98" s="2"/>
+      <x:c r="C98" s="2"/>
+      <x:c r="D98" s="2"/>
+      <x:c r="E98" s="2"/>
+      <x:c r="F98" s="2"/>
+      <x:c r="G98" s="2"/>
+      <x:c r="H98" s="2"/>
+      <x:c r="I98" s="2"/>
+      <x:c r="J98" s="2"/>
+      <x:c r="K98" s="2"/>
+      <x:c r="L98" s="2"/>
+      <x:c r="M98" s="2"/>
+      <x:c r="N98" s="2"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="2"/>
+      <x:c r="B99" s="2"/>
+      <x:c r="C99" s="2"/>
+      <x:c r="D99" s="2"/>
+      <x:c r="E99" s="2"/>
+      <x:c r="F99" s="2"/>
+      <x:c r="G99" s="2"/>
+      <x:c r="H99" s="2"/>
+      <x:c r="I99" s="2"/>
+      <x:c r="J99" s="2"/>
+      <x:c r="K99" s="2"/>
+      <x:c r="L99" s="2"/>
+      <x:c r="M99" s="2"/>
+      <x:c r="N99" s="2"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="2"/>
+      <x:c r="B100" s="2"/>
+      <x:c r="C100" s="2"/>
+      <x:c r="D100" s="2"/>
+      <x:c r="E100" s="2"/>
+      <x:c r="F100" s="2"/>
+      <x:c r="G100" s="2"/>
+      <x:c r="H100" s="2"/>
+      <x:c r="I100" s="2"/>
+      <x:c r="J100" s="2"/>
+      <x:c r="K100" s="2"/>
+      <x:c r="L100" s="2"/>
+      <x:c r="M100" s="2"/>
+      <x:c r="N100" s="2"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="2"/>
+      <x:c r="B101" s="2"/>
+      <x:c r="C101" s="2"/>
+      <x:c r="D101" s="2"/>
+      <x:c r="E101" s="2"/>
+      <x:c r="F101" s="2"/>
+      <x:c r="G101" s="2"/>
+      <x:c r="H101" s="2"/>
+      <x:c r="I101" s="2"/>
+      <x:c r="J101" s="2"/>
+      <x:c r="K101" s="2"/>
+      <x:c r="L101" s="2"/>
+      <x:c r="M101" s="2"/>
+      <x:c r="N101" s="2"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="2"/>
+      <x:c r="B102" s="2"/>
+      <x:c r="C102" s="2"/>
+      <x:c r="D102" s="2"/>
+      <x:c r="E102" s="2"/>
+      <x:c r="F102" s="2"/>
+      <x:c r="G102" s="2"/>
+      <x:c r="H102" s="2"/>
+      <x:c r="I102" s="2"/>
+      <x:c r="J102" s="2"/>
+      <x:c r="K102" s="2"/>
+      <x:c r="L102" s="2"/>
+      <x:c r="M102" s="2"/>
+      <x:c r="N102" s="2"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="2"/>
+      <x:c r="B103" s="2"/>
+      <x:c r="C103" s="2"/>
+      <x:c r="D103" s="2"/>
+      <x:c r="E103" s="2"/>
+      <x:c r="F103" s="2"/>
+      <x:c r="G103" s="2"/>
+      <x:c r="H103" s="2"/>
+      <x:c r="I103" s="2"/>
+      <x:c r="J103" s="2"/>
+      <x:c r="K103" s="2"/>
+      <x:c r="L103" s="2"/>
+      <x:c r="M103" s="2"/>
+      <x:c r="N103" s="2"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="2"/>
+      <x:c r="B104" s="2"/>
+      <x:c r="C104" s="2"/>
+      <x:c r="D104" s="2"/>
+      <x:c r="E104" s="2"/>
+      <x:c r="F104" s="2"/>
+      <x:c r="G104" s="2"/>
+      <x:c r="H104" s="2"/>
+      <x:c r="I104" s="2"/>
+      <x:c r="J104" s="2"/>
+      <x:c r="K104" s="2"/>
+      <x:c r="L104" s="2"/>
+      <x:c r="M104" s="2"/>
+      <x:c r="N104" s="2"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="2"/>
+      <x:c r="B105" s="2"/>
+      <x:c r="C105" s="2"/>
+      <x:c r="D105" s="2"/>
+      <x:c r="E105" s="2"/>
+      <x:c r="F105" s="2"/>
+      <x:c r="G105" s="2"/>
+      <x:c r="H105" s="2"/>
+      <x:c r="I105" s="2"/>
+      <x:c r="J105" s="2"/>
+      <x:c r="K105" s="2"/>
+      <x:c r="L105" s="2"/>
+      <x:c r="M105" s="2"/>
+      <x:c r="N105" s="2"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="2"/>
+      <x:c r="B106" s="2"/>
+      <x:c r="C106" s="2"/>
+      <x:c r="D106" s="2"/>
+      <x:c r="E106" s="2"/>
+      <x:c r="F106" s="2"/>
+      <x:c r="G106" s="2"/>
+      <x:c r="H106" s="2"/>
+      <x:c r="I106" s="2"/>
+      <x:c r="J106" s="2"/>
+      <x:c r="K106" s="2"/>
+      <x:c r="L106" s="2"/>
+      <x:c r="M106" s="2"/>
+      <x:c r="N106" s="2"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="2"/>
+      <x:c r="B107" s="2"/>
+      <x:c r="C107" s="2"/>
+      <x:c r="D107" s="2"/>
+      <x:c r="E107" s="2"/>
+      <x:c r="F107" s="2"/>
+      <x:c r="G107" s="2"/>
+      <x:c r="H107" s="2"/>
+      <x:c r="I107" s="2"/>
+      <x:c r="J107" s="2"/>
+      <x:c r="K107" s="2"/>
+      <x:c r="L107" s="2"/>
+      <x:c r="M107" s="2"/>
+      <x:c r="N107" s="2"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="2"/>
+      <x:c r="B108" s="2"/>
+      <x:c r="C108" s="2"/>
+      <x:c r="D108" s="2"/>
+      <x:c r="E108" s="2"/>
+      <x:c r="F108" s="2"/>
+      <x:c r="G108" s="2"/>
+      <x:c r="H108" s="2"/>
+      <x:c r="I108" s="2"/>
+      <x:c r="J108" s="2"/>
+      <x:c r="K108" s="2"/>
+      <x:c r="L108" s="2"/>
+      <x:c r="M108" s="2"/>
+      <x:c r="N108" s="2"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="2"/>
+      <x:c r="B109" s="2"/>
+      <x:c r="C109" s="2"/>
+      <x:c r="D109" s="2"/>
+      <x:c r="E109" s="2"/>
+      <x:c r="F109" s="2"/>
+      <x:c r="G109" s="2"/>
+      <x:c r="H109" s="2"/>
+      <x:c r="I109" s="2"/>
+      <x:c r="J109" s="2"/>
+      <x:c r="K109" s="2"/>
+      <x:c r="L109" s="2"/>
+      <x:c r="M109" s="2"/>
+      <x:c r="N109" s="2"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="2"/>
+      <x:c r="B110" s="2"/>
+      <x:c r="C110" s="2"/>
+      <x:c r="D110" s="2"/>
+      <x:c r="E110" s="2"/>
+      <x:c r="F110" s="2"/>
+      <x:c r="G110" s="2"/>
+      <x:c r="H110" s="2"/>
+      <x:c r="I110" s="2"/>
+      <x:c r="J110" s="2"/>
+      <x:c r="K110" s="2"/>
+      <x:c r="L110" s="2"/>
+      <x:c r="M110" s="2"/>
+      <x:c r="N110" s="2"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="2"/>
+      <x:c r="B111" s="2"/>
+      <x:c r="C111" s="2"/>
+      <x:c r="D111" s="2"/>
+      <x:c r="E111" s="2"/>
+      <x:c r="F111" s="2"/>
+      <x:c r="G111" s="2"/>
+      <x:c r="H111" s="2"/>
+      <x:c r="I111" s="2"/>
+      <x:c r="J111" s="2"/>
+      <x:c r="K111" s="2"/>
+      <x:c r="L111" s="2"/>
+      <x:c r="M111" s="2"/>
+      <x:c r="N111" s="2"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="2"/>
+      <x:c r="B112" s="2"/>
+      <x:c r="C112" s="2"/>
+      <x:c r="D112" s="2"/>
+      <x:c r="E112" s="2"/>
+      <x:c r="F112" s="2"/>
+      <x:c r="G112" s="2"/>
+      <x:c r="H112" s="2"/>
+      <x:c r="I112" s="2"/>
+      <x:c r="J112" s="2"/>
+      <x:c r="K112" s="2"/>
+      <x:c r="L112" s="2"/>
+      <x:c r="M112" s="2"/>
+      <x:c r="N112" s="2"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="2"/>
+      <x:c r="B113" s="2"/>
+      <x:c r="C113" s="2"/>
+      <x:c r="D113" s="2"/>
+      <x:c r="E113" s="2"/>
+      <x:c r="F113" s="2"/>
+      <x:c r="G113" s="2"/>
+      <x:c r="H113" s="2"/>
+      <x:c r="I113" s="2"/>
+      <x:c r="J113" s="2"/>
+      <x:c r="K113" s="2"/>
+      <x:c r="L113" s="2"/>
+      <x:c r="M113" s="2"/>
+      <x:c r="N113" s="2"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="2"/>
+      <x:c r="B114" s="2"/>
+      <x:c r="C114" s="2"/>
+      <x:c r="D114" s="2"/>
+      <x:c r="E114" s="2"/>
+      <x:c r="F114" s="2"/>
+      <x:c r="G114" s="2"/>
+      <x:c r="H114" s="2"/>
+      <x:c r="I114" s="2"/>
+      <x:c r="J114" s="2"/>
+      <x:c r="K114" s="2"/>
+      <x:c r="L114" s="2"/>
+      <x:c r="M114" s="2"/>
+      <x:c r="N114" s="2"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="2"/>
+      <x:c r="B115" s="2"/>
+      <x:c r="C115" s="2"/>
+      <x:c r="D115" s="2"/>
+      <x:c r="E115" s="2"/>
+      <x:c r="F115" s="2"/>
+      <x:c r="G115" s="2"/>
+      <x:c r="H115" s="2"/>
+      <x:c r="I115" s="2"/>
+      <x:c r="J115" s="2"/>
+      <x:c r="K115" s="2"/>
+      <x:c r="L115" s="2"/>
+      <x:c r="M115" s="2"/>
+      <x:c r="N115" s="2"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="2"/>
+      <x:c r="B116" s="2"/>
+      <x:c r="C116" s="2"/>
+      <x:c r="D116" s="2"/>
+      <x:c r="E116" s="2"/>
+      <x:c r="F116" s="2"/>
+      <x:c r="G116" s="2"/>
+      <x:c r="H116" s="2"/>
+      <x:c r="I116" s="2"/>
+      <x:c r="J116" s="2"/>
+      <x:c r="K116" s="2"/>
+      <x:c r="L116" s="2"/>
+      <x:c r="M116" s="2"/>
+      <x:c r="N116" s="2"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="2"/>
+      <x:c r="B117" s="2"/>
+      <x:c r="C117" s="2"/>
+      <x:c r="D117" s="2"/>
+      <x:c r="E117" s="2"/>
+      <x:c r="F117" s="2"/>
+      <x:c r="G117" s="2"/>
+      <x:c r="H117" s="2"/>
+      <x:c r="I117" s="2"/>
+      <x:c r="J117" s="2"/>
+      <x:c r="K117" s="2"/>
+      <x:c r="L117" s="2"/>
+      <x:c r="M117" s="2"/>
+      <x:c r="N117" s="2"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="2"/>
+      <x:c r="B118" s="2"/>
+      <x:c r="C118" s="2"/>
+      <x:c r="D118" s="2"/>
+      <x:c r="E118" s="2"/>
+      <x:c r="F118" s="2"/>
+      <x:c r="G118" s="2"/>
+      <x:c r="H118" s="2"/>
+      <x:c r="I118" s="2"/>
+      <x:c r="J118" s="2"/>
+      <x:c r="K118" s="2"/>
+      <x:c r="L118" s="2"/>
+      <x:c r="M118" s="2"/>
+      <x:c r="N118" s="2"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="2"/>
+      <x:c r="B119" s="2"/>
+      <x:c r="C119" s="2"/>
+      <x:c r="D119" s="2"/>
+      <x:c r="E119" s="2"/>
+      <x:c r="F119" s="2"/>
+      <x:c r="G119" s="2"/>
+      <x:c r="H119" s="2"/>
+      <x:c r="I119" s="2"/>
+      <x:c r="J119" s="2"/>
+      <x:c r="K119" s="2"/>
+      <x:c r="L119" s="2"/>
+      <x:c r="M119" s="2"/>
+      <x:c r="N119" s="2"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="2"/>
+      <x:c r="B120" s="2"/>
+      <x:c r="C120" s="2"/>
+      <x:c r="D120" s="2"/>
+      <x:c r="E120" s="2"/>
+      <x:c r="F120" s="2"/>
+      <x:c r="G120" s="2"/>
+      <x:c r="H120" s="2"/>
+      <x:c r="I120" s="2"/>
+      <x:c r="J120" s="2"/>
+      <x:c r="K120" s="2"/>
+      <x:c r="L120" s="2"/>
+      <x:c r="M120" s="2"/>
+      <x:c r="N120" s="2"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="2"/>
+      <x:c r="B121" s="2"/>
+      <x:c r="C121" s="2"/>
+      <x:c r="D121" s="2"/>
+      <x:c r="E121" s="2"/>
+      <x:c r="F121" s="2"/>
+      <x:c r="G121" s="2"/>
+      <x:c r="H121" s="2"/>
+      <x:c r="I121" s="2"/>
+      <x:c r="J121" s="2"/>
+      <x:c r="K121" s="2"/>
+      <x:c r="L121" s="2"/>
+      <x:c r="M121" s="2"/>
+      <x:c r="N121" s="2"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="2"/>
+      <x:c r="B122" s="2"/>
+      <x:c r="C122" s="2"/>
+      <x:c r="D122" s="2"/>
+      <x:c r="E122" s="2"/>
+      <x:c r="F122" s="2"/>
+      <x:c r="G122" s="2"/>
+      <x:c r="H122" s="2"/>
+      <x:c r="I122" s="2"/>
+      <x:c r="J122" s="2"/>
+      <x:c r="K122" s="2"/>
+      <x:c r="L122" s="2"/>
+      <x:c r="M122" s="2"/>
+      <x:c r="N122" s="2"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="2"/>
+      <x:c r="B123" s="2"/>
+      <x:c r="C123" s="2"/>
+      <x:c r="D123" s="2"/>
+      <x:c r="E123" s="2"/>
+      <x:c r="F123" s="2"/>
+      <x:c r="G123" s="2"/>
+      <x:c r="H123" s="2"/>
+      <x:c r="I123" s="2"/>
+      <x:c r="J123" s="2"/>
+      <x:c r="K123" s="2"/>
+      <x:c r="L123" s="2"/>
+      <x:c r="M123" s="2"/>
+      <x:c r="N123" s="2"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="2"/>
+      <x:c r="B124" s="2"/>
+      <x:c r="C124" s="2"/>
+      <x:c r="D124" s="2"/>
+      <x:c r="E124" s="2"/>
+      <x:c r="F124" s="2"/>
+      <x:c r="G124" s="2"/>
+      <x:c r="H124" s="2"/>
+      <x:c r="I124" s="2"/>
+      <x:c r="J124" s="2"/>
+      <x:c r="K124" s="2"/>
+      <x:c r="L124" s="2"/>
+      <x:c r="M124" s="2"/>
+      <x:c r="N124" s="2"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="2"/>
+      <x:c r="B125" s="2"/>
+      <x:c r="C125" s="2"/>
+      <x:c r="D125" s="2"/>
+      <x:c r="E125" s="2"/>
+      <x:c r="F125" s="2"/>
+      <x:c r="G125" s="2"/>
+      <x:c r="H125" s="2"/>
+      <x:c r="I125" s="2"/>
+      <x:c r="J125" s="2"/>
+      <x:c r="K125" s="2"/>
+      <x:c r="L125" s="2"/>
+      <x:c r="M125" s="2"/>
+      <x:c r="N125" s="2"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="2"/>
+      <x:c r="B126" s="2"/>
+      <x:c r="C126" s="2"/>
+      <x:c r="D126" s="2"/>
+      <x:c r="E126" s="2"/>
+      <x:c r="F126" s="2"/>
+      <x:c r="G126" s="2"/>
+      <x:c r="H126" s="2"/>
+      <x:c r="I126" s="2"/>
+      <x:c r="J126" s="2"/>
+      <x:c r="K126" s="2"/>
+      <x:c r="L126" s="2"/>
+      <x:c r="M126" s="2"/>
+      <x:c r="N126" s="2"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="2"/>
+      <x:c r="B127" s="2"/>
+      <x:c r="C127" s="2"/>
+      <x:c r="D127" s="2"/>
+      <x:c r="E127" s="2"/>
+      <x:c r="F127" s="2"/>
+      <x:c r="G127" s="2"/>
+      <x:c r="H127" s="2"/>
+      <x:c r="I127" s="2"/>
+      <x:c r="J127" s="2"/>
+      <x:c r="K127" s="2"/>
+      <x:c r="L127" s="2"/>
+      <x:c r="M127" s="2"/>
+      <x:c r="N127" s="2"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="2"/>
+      <x:c r="B128" s="2"/>
+      <x:c r="C128" s="2"/>
+      <x:c r="D128" s="2"/>
+      <x:c r="E128" s="2"/>
+      <x:c r="F128" s="2"/>
+      <x:c r="G128" s="2"/>
+      <x:c r="H128" s="2"/>
+      <x:c r="I128" s="2"/>
+      <x:c r="J128" s="2"/>
+      <x:c r="K128" s="2"/>
+      <x:c r="L128" s="2"/>
+      <x:c r="M128" s="2"/>
+      <x:c r="N128" s="2"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="2"/>
+      <x:c r="B129" s="2"/>
+      <x:c r="C129" s="2"/>
+      <x:c r="D129" s="2"/>
+      <x:c r="E129" s="2"/>
+      <x:c r="F129" s="2"/>
+      <x:c r="G129" s="2"/>
+      <x:c r="H129" s="2"/>
+      <x:c r="I129" s="2"/>
+      <x:c r="J129" s="2"/>
+      <x:c r="K129" s="2"/>
+      <x:c r="L129" s="2"/>
+      <x:c r="M129" s="2"/>
+      <x:c r="N129" s="2"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="2"/>
+      <x:c r="B130" s="2"/>
+      <x:c r="C130" s="2"/>
+      <x:c r="D130" s="2"/>
+      <x:c r="E130" s="2"/>
+      <x:c r="F130" s="2"/>
+      <x:c r="G130" s="2"/>
+      <x:c r="H130" s="2"/>
+      <x:c r="I130" s="2"/>
+      <x:c r="J130" s="2"/>
+      <x:c r="K130" s="2"/>
+      <x:c r="L130" s="2"/>
+      <x:c r="M130" s="2"/>
+      <x:c r="N130" s="2"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="2"/>
+      <x:c r="B131" s="2"/>
+      <x:c r="C131" s="2"/>
+      <x:c r="D131" s="2"/>
+      <x:c r="E131" s="2"/>
+      <x:c r="F131" s="2"/>
+      <x:c r="G131" s="2"/>
+      <x:c r="H131" s="2"/>
+      <x:c r="I131" s="2"/>
+      <x:c r="J131" s="2"/>
+      <x:c r="K131" s="2"/>
+      <x:c r="L131" s="2"/>
+      <x:c r="M131" s="2"/>
+      <x:c r="N131" s="2"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="2"/>
+      <x:c r="B132" s="2"/>
+      <x:c r="C132" s="2"/>
+      <x:c r="D132" s="2"/>
+      <x:c r="E132" s="2"/>
+      <x:c r="F132" s="2"/>
+      <x:c r="G132" s="2"/>
+      <x:c r="H132" s="2"/>
+      <x:c r="I132" s="2"/>
+      <x:c r="J132" s="2"/>
+      <x:c r="K132" s="2"/>
+      <x:c r="L132" s="2"/>
+      <x:c r="M132" s="2"/>
+      <x:c r="N132" s="2"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="2"/>
+      <x:c r="B133" s="2"/>
+      <x:c r="C133" s="2"/>
+      <x:c r="D133" s="2"/>
+      <x:c r="E133" s="2"/>
+      <x:c r="F133" s="2"/>
+      <x:c r="G133" s="2"/>
+      <x:c r="H133" s="2"/>
+      <x:c r="I133" s="2"/>
+      <x:c r="J133" s="2"/>
+      <x:c r="K133" s="2"/>
+      <x:c r="L133" s="2"/>
+      <x:c r="M133" s="2"/>
+      <x:c r="N133" s="2"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="2"/>
+      <x:c r="B134" s="2"/>
+      <x:c r="C134" s="2"/>
+      <x:c r="D134" s="2"/>
+      <x:c r="E134" s="2"/>
+      <x:c r="F134" s="2"/>
+      <x:c r="G134" s="2"/>
+      <x:c r="H134" s="2"/>
+      <x:c r="I134" s="2"/>
+      <x:c r="J134" s="2"/>
+      <x:c r="K134" s="2"/>
+      <x:c r="L134" s="2"/>
+      <x:c r="M134" s="2"/>
+      <x:c r="N134" s="2"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="2"/>
+      <x:c r="B135" s="2"/>
+      <x:c r="C135" s="2"/>
+      <x:c r="D135" s="2"/>
+      <x:c r="E135" s="2"/>
+      <x:c r="F135" s="2"/>
+      <x:c r="G135" s="2"/>
+      <x:c r="H135" s="2"/>
+      <x:c r="I135" s="2"/>
+      <x:c r="J135" s="2"/>
+      <x:c r="K135" s="2"/>
+      <x:c r="L135" s="2"/>
+      <x:c r="M135" s="2"/>
+      <x:c r="N135" s="2"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="2"/>
+      <x:c r="B136" s="2"/>
+      <x:c r="C136" s="2"/>
+      <x:c r="D136" s="2"/>
+      <x:c r="E136" s="2"/>
+      <x:c r="F136" s="2"/>
+      <x:c r="G136" s="2"/>
+      <x:c r="H136" s="2"/>
+      <x:c r="I136" s="2"/>
+      <x:c r="J136" s="2"/>
+      <x:c r="K136" s="2"/>
+      <x:c r="L136" s="2"/>
+      <x:c r="M136" s="2"/>
+      <x:c r="N136" s="2"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="2"/>
+      <x:c r="B137" s="2"/>
+      <x:c r="C137" s="2"/>
+      <x:c r="D137" s="2"/>
+      <x:c r="E137" s="2"/>
+      <x:c r="F137" s="2"/>
+      <x:c r="G137" s="2"/>
+      <x:c r="H137" s="2"/>
+      <x:c r="I137" s="2"/>
+      <x:c r="J137" s="2"/>
+      <x:c r="K137" s="2"/>
+      <x:c r="L137" s="2"/>
+      <x:c r="M137" s="2"/>
+      <x:c r="N137" s="2"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="2"/>
+      <x:c r="B138" s="2"/>
+      <x:c r="C138" s="2"/>
+      <x:c r="D138" s="2"/>
+      <x:c r="E138" s="2"/>
+      <x:c r="F138" s="2"/>
+      <x:c r="G138" s="2"/>
+      <x:c r="H138" s="2"/>
+      <x:c r="I138" s="2"/>
+      <x:c r="J138" s="2"/>
+      <x:c r="K138" s="2"/>
+      <x:c r="L138" s="2"/>
+      <x:c r="M138" s="2"/>
+      <x:c r="N138" s="2"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="2"/>
+      <x:c r="B139" s="2"/>
+      <x:c r="C139" s="2"/>
+      <x:c r="D139" s="2"/>
+      <x:c r="E139" s="2"/>
+      <x:c r="F139" s="2"/>
+      <x:c r="G139" s="2"/>
+      <x:c r="H139" s="2"/>
+      <x:c r="I139" s="2"/>
+      <x:c r="J139" s="2"/>
+      <x:c r="K139" s="2"/>
+      <x:c r="L139" s="2"/>
+      <x:c r="M139" s="2"/>
+      <x:c r="N139" s="2"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="2"/>
+      <x:c r="B140" s="2"/>
+      <x:c r="C140" s="2"/>
+      <x:c r="D140" s="2"/>
+      <x:c r="E140" s="2"/>
+      <x:c r="F140" s="2"/>
+      <x:c r="G140" s="2"/>
+      <x:c r="H140" s="2"/>
+      <x:c r="I140" s="2"/>
+      <x:c r="J140" s="2"/>
+      <x:c r="K140" s="2"/>
+      <x:c r="L140" s="2"/>
+      <x:c r="M140" s="2"/>
+      <x:c r="N140" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52ab6eafdcc40bb"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16.25" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Checks</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+      <x:c r="G1" s="2"/>
+      <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Sanity checks：公式、来源、口径和空值。</x:v>
+      </x:c>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+      <x:c r="J2" s="2"/>
+      <x:c r="K2" s="2"/>
+      <x:c r="L2" s="2"/>
+      <x:c r="M2" s="2"/>
+      <x:c r="N2" s="2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+      <x:c r="J3" s="2"/>
+      <x:c r="K3" s="2"/>
+      <x:c r="L3" s="2"/>
+      <x:c r="M3" s="2"/>
+      <x:c r="N3" s="2"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="7" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>Formula result</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
+      <x:c r="J4" s="2"/>
+      <x:c r="K4" s="2"/>
+      <x:c r="L4" s="2"/>
+      <x:c r="M4" s="2"/>
+      <x:c r="N4" s="2"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="str">
+        <x:v>Q1 revenue YoY ties to release</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="b">
+        <x:f>ABS(('Financials KPIs'!H5/'Financials KPIs'!G5-1)-0.236)&lt;0.02</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:f>IF(B5,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>Expected about 24%</x:v>
+      </x:c>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
+      <x:c r="I5" s="2"/>
+      <x:c r="J5" s="2"/>
+      <x:c r="K5" s="2"/>
+      <x:c r="L5" s="2"/>
+      <x:c r="M5" s="2"/>
+      <x:c r="N5" s="2"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="2" t="str">
+        <x:v>Gross margin recalculates from Q1 revenue/gross profit</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="b">
+        <x:f>ABS(('Financials KPIs'!H6/'Financials KPIs'!H5*100)-'Financials KPIs'!H7)&lt;0.1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:f>IF(B6,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>Q1 2026 gross margin should be about 46.6%</x:v>
+      </x:c>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
+      <x:c r="I6" s="2"/>
+      <x:c r="J6" s="2"/>
+      <x:c r="K6" s="2"/>
+      <x:c r="L6" s="2"/>
+      <x:c r="M6" s="2"/>
+      <x:c r="N6" s="2"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="str">
+        <x:v>EV equals market cap minus net cash</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="b">
+        <x:f>ABS(Valuation!B9-(Valuation!B7-Valuation!B8))&lt;0.01</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:f>IF(B7,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D7" s="2" t="str">
+        <x:v>Valuation formula cross-check</x:v>
+      </x:c>
+      <x:c r="E7" s="2"/>
+      <x:c r="F7" s="2"/>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
+      <x:c r="I7" s="2"/>
+      <x:c r="J7" s="2"/>
+      <x:c r="K7" s="2"/>
+      <x:c r="L7" s="2"/>
+      <x:c r="M7" s="2"/>
+      <x:c r="N7" s="2"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="str">
+        <x:v>Backlog ASP equals backlog value / backlog GW</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="b">
+        <x:f>ABS(Valuation!B18-(Valuation!B17/Valuation!B16))&lt;0.001</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:f>IF(B8,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D8" s="2" t="str">
+        <x:v>Backlog value is USD bn; GW maps to $/W</x:v>
+      </x:c>
+      <x:c r="E8" s="2"/>
+      <x:c r="F8" s="2"/>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2"/>
+      <x:c r="I8" s="2"/>
+      <x:c r="J8" s="2"/>
+      <x:c r="K8" s="2"/>
+      <x:c r="L8" s="2"/>
+      <x:c r="M8" s="2"/>
+      <x:c r="N8" s="2"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="str">
+        <x:v>Source count &gt;= 12</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="b">
+        <x:f>COUNTA(Sources!A5:A50)&gt;=12</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:f>IF(B9,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>Coverage and citation sanity check</x:v>
+      </x:c>
+      <x:c r="E9" s="2"/>
+      <x:c r="F9" s="2"/>
+      <x:c r="G9" s="2"/>
+      <x:c r="H9" s="2"/>
+      <x:c r="I9" s="2"/>
+      <x:c r="J9" s="2"/>
+      <x:c r="K9" s="2"/>
+      <x:c r="L9" s="2"/>
+      <x:c r="M9" s="2"/>
+      <x:c r="N9" s="2"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="str">
+        <x:v>Critical valuation inputs are nonblank</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="b">
+        <x:f>COUNTBLANK(Valuation!B5:B18)=0</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:f>IF(B10,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>Avoid silent blank-driven formulas</x:v>
+      </x:c>
+      <x:c r="E10" s="2"/>
+      <x:c r="F10" s="2"/>
+      <x:c r="G10" s="2"/>
+      <x:c r="H10" s="2"/>
+      <x:c r="I10" s="2"/>
+      <x:c r="J10" s="2"/>
+      <x:c r="K10" s="2"/>
+      <x:c r="L10" s="2"/>
+      <x:c r="M10" s="2"/>
+      <x:c r="N10" s="2"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="str">
+        <x:v>Market reaction alpha formula ties</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="b">
+        <x:f>ABS('Market Reaction'!N5-('Market Reaction'!I5-'Market Reaction'!J5))&lt;0.01</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:f>IF(B11,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>alpha = FSLR return - TAN return</x:v>
+      </x:c>
+      <x:c r="E11" s="2"/>
+      <x:c r="F11" s="2"/>
+      <x:c r="G11" s="2"/>
+      <x:c r="H11" s="2"/>
+      <x:c r="I11" s="2"/>
+      <x:c r="J11" s="2"/>
+      <x:c r="K11" s="2"/>
+      <x:c r="L11" s="2"/>
+      <x:c r="M11" s="2"/>
+      <x:c r="N11" s="2"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="str">
+        <x:v>FY2026 EBITDA midpoint is $2.7bn</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="b">
+        <x:f>ABS(Valuation!B11-2.7)&lt;0.001</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:f>IF(B12,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>From $2.6-$2.8bn guidance</x:v>
+      </x:c>
+      <x:c r="E12" s="2"/>
+      <x:c r="F12" s="2"/>
+      <x:c r="G12" s="2"/>
+      <x:c r="H12" s="2"/>
+      <x:c r="I12" s="2"/>
+      <x:c r="J12" s="2"/>
+      <x:c r="K12" s="2"/>
+      <x:c r="L12" s="2"/>
+      <x:c r="M12" s="2"/>
+      <x:c r="N12" s="2"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2"/>
+      <x:c r="B13" s="2"/>
+      <x:c r="C13" s="2"/>
+      <x:c r="D13" s="2"/>
+      <x:c r="E13" s="2"/>
+      <x:c r="F13" s="2"/>
+      <x:c r="G13" s="2"/>
+      <x:c r="H13" s="2"/>
+      <x:c r="I13" s="2"/>
+      <x:c r="J13" s="2"/>
+      <x:c r="K13" s="2"/>
+      <x:c r="L13" s="2"/>
+      <x:c r="M13" s="2"/>
+      <x:c r="N13" s="2"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="2"/>
+      <x:c r="C14" s="2"/>
+      <x:c r="D14" s="2"/>
+      <x:c r="E14" s="2"/>
+      <x:c r="F14" s="2"/>
+      <x:c r="G14" s="2"/>
+      <x:c r="H14" s="2"/>
+      <x:c r="I14" s="2"/>
+      <x:c r="J14" s="2"/>
+      <x:c r="K14" s="2"/>
+      <x:c r="L14" s="2"/>
+      <x:c r="M14" s="2"/>
+      <x:c r="N14" s="2"/>
+    </x:row>
+    <x:row r="15">
       <x:c r="A15" s="2"/>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2" t="str">
-        <x:v>Bull</x:v>
-      </x:c>
-      <x:c r="E15" s="15" t="n">
-        <x:v>375.4200250894393</x:v>
-      </x:c>
-      <x:c r="F15" s="16" t="n">
-        <x:f>E15/Valuation!$B$5-1</x:f>
-        <x:v>0.29681004884173934</x:v>
-      </x:c>
+      <x:c r="D15" s="2"/>
+      <x:c r="E15" s="2"/>
+      <x:c r="F15" s="2"/>
       <x:c r="G15" s="2"/>
       <x:c r="H15" s="2"/>
       <x:c r="I15" s="2"/>
@@ -3694,7 +6080,6 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32e0a21d549e4c40"/>
 </x:worksheet>
 </file>
 
@@ -6318,9 +8703,9 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0816eaed3e6c4660"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaa8148f25024091"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2187e4cc8d854a1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5956d8a64d24719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6432,7 +8817,7 @@
         <x:v>Current price</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>289.495</x:v>
+        <x:v>294.41</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
         <x:v>USD/share</x:v>
@@ -6495,7 +8880,7 @@
       </x:c>
       <x:c r="B7" s="22" t="n">
         <x:f>B5*B6/1000</x:f>
-        <x:v>31.154004425</x:v>
+        <x:v>31.68293215</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
         <x:v>USD bn</x:v>
@@ -6553,7 +8938,7 @@
       </x:c>
       <x:c r="B9" s="22" t="n">
         <x:f>B7-B8</x:f>
-        <x:v>29.153178425</x:v>
+        <x:v>29.68210615</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
         <x:v>USD bn</x:v>
@@ -6658,7 +9043,7 @@
       </x:c>
       <x:c r="B13" s="22" t="n">
         <x:f>B5/B12</x:f>
-        <x:v>18.701227390180875</x:v>
+        <x:v>19.0187338501292</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>x</x:v>
@@ -6685,7 +9070,7 @@
       </x:c>
       <x:c r="B14" s="22" t="n">
         <x:f>B9/B10</x:f>
-        <x:v>5.772906618811882</x:v>
+        <x:v>5.877644782178218</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>x</x:v>
@@ -6712,7 +9097,7 @@
       </x:c>
       <x:c r="B15" s="22" t="n">
         <x:f>B9/B11</x:f>
-        <x:v>10.79747349074074</x:v>
+        <x:v>10.993372648148148</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
         <x:v>x</x:v>
@@ -8828,7 +11213,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8966cc05e05145ef"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fdc81339f5f4d3b"/>
 </x:worksheet>
 </file>
 
@@ -8872,7 +11257,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>同行估值快照；FSLR 同时给出公司口径 cross-check。</x:v>
+        <x:v>Solar ecosystem directional comparison only; FSLR uses company-basis EV and deserves separate treatment because of CdTe, U.S. manufacturing, backlog and 45X sensitivity.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -8974,28 +11359,28 @@
         <x:v>CdTe modules, U.S. manufacturing</x:v>
       </x:c>
       <x:c r="D5" s="30" t="n">
-        <x:v>289.495</x:v>
+        <x:v>294.41</x:v>
       </x:c>
       <x:c r="E5" s="30" t="n">
-        <x:v>31.16</x:v>
+        <x:v>31.68</x:v>
       </x:c>
       <x:c r="F5" s="30" t="n">
-        <x:v>27.57</x:v>
+        <x:v>29.68</x:v>
       </x:c>
       <x:c r="G5" s="30" t="n">
-        <x:v>18.74</x:v>
+        <x:v>19.02</x:v>
       </x:c>
       <x:c r="H5" s="30" t="n">
-        <x:v>15.08</x:v>
+        <x:v>15.27</x:v>
       </x:c>
       <x:c r="I5" s="30" t="n">
-        <x:v>5.43</x:v>
+        <x:v>5.89</x:v>
       </x:c>
       <x:c r="J5" s="30" t="n">
-        <x:v>5.09</x:v>
+        <x:v>5.48</x:v>
       </x:c>
       <x:c r="K5" s="30" t="n">
-        <x:v>12.13</x:v>
+        <x:v>13.23</x:v>
       </x:c>
       <x:c r="L5" s="30" t="str">
         <x:v>S12</x:v>
@@ -9004,22 +11389,22 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N5" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>FSLR market cap/EV/PE use company-basis current price, Q1 diluted shares and Q1 net cash; peer multiples are directional only.</x:v>
       </x:c>
       <x:c r="O5" s="31" t="n">
-        <x:v>31.15</x:v>
+        <x:v>31.68</x:v>
       </x:c>
       <x:c r="P5" s="31" t="n">
-        <x:v>29.15</x:v>
+        <x:v>29.68</x:v>
       </x:c>
       <x:c r="Q5" s="31" t="n">
-        <x:v>18.7</x:v>
+        <x:v>19.02</x:v>
       </x:c>
       <x:c r="R5" s="29" t="n">
-        <x:v>5.77</x:v>
+        <x:v>5.88</x:v>
       </x:c>
       <x:c r="S5" s="29" t="n">
-        <x:v>10.8</x:v>
+        <x:v>10.99</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9033,28 +11418,28 @@
         <x:v>microinverters/storage</x:v>
       </x:c>
       <x:c r="D6" s="30" t="n">
-        <x:v>68.981</x:v>
+        <x:v>70.478</x:v>
       </x:c>
       <x:c r="E6" s="30" t="n">
-        <x:v>9.11</x:v>
+        <x:v>9.29</x:v>
       </x:c>
       <x:c r="F6" s="30" t="n">
-        <x:v>8.94</x:v>
+        <x:v>9.07</x:v>
       </x:c>
       <x:c r="G6" s="30" t="n">
-        <x:v>67.73</x:v>
+        <x:v>68.95</x:v>
       </x:c>
       <x:c r="H6" s="30" t="n">
-        <x:v>33.91</x:v>
+        <x:v>34.52</x:v>
       </x:c>
       <x:c r="I6" s="30" t="n">
-        <x:v>6.62</x:v>
+        <x:v>6.71</x:v>
       </x:c>
       <x:c r="J6" s="30" t="n">
-        <x:v>6.39</x:v>
+        <x:v>6.48</x:v>
       </x:c>
       <x:c r="K6" s="30" t="n">
-        <x:v>49.92</x:v>
+        <x:v>50.64</x:v>
       </x:c>
       <x:c r="L6" s="30" t="str">
         <x:v>S12</x:v>
@@ -9063,7 +11448,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N6" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O6" s="31" t="str"/>
       <x:c r="P6" s="31" t="str"/>
@@ -9082,17 +11467,17 @@
         <x:v>inverters/optimizer</x:v>
       </x:c>
       <x:c r="D7" s="30" t="n">
-        <x:v>71.7</x:v>
+        <x:v>72.67</x:v>
       </x:c>
       <x:c r="E7" s="30" t="n">
-        <x:v>4.42</x:v>
+        <x:v>4.39</x:v>
       </x:c>
       <x:c r="F7" s="30" t="n">
         <x:v>4.32</x:v>
       </x:c>
       <x:c r="G7" s="30" t="str"/>
       <x:c r="H7" s="30" t="n">
-        <x:v>123.83</x:v>
+        <x:v>123.08</x:v>
       </x:c>
       <x:c r="I7" s="30" t="n">
         <x:v>3.49</x:v>
@@ -9108,7 +11493,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O7" s="31" t="str"/>
       <x:c r="P7" s="31" t="str"/>
@@ -9127,10 +11512,10 @@
         <x:v>modules/projects/storage</x:v>
       </x:c>
       <x:c r="D8" s="30" t="n">
-        <x:v>19.69</x:v>
+        <x:v>20.01</x:v>
       </x:c>
       <x:c r="E8" s="30" t="n">
-        <x:v>1.32</x:v>
+        <x:v>1.35</x:v>
       </x:c>
       <x:c r="F8" s="30" t="n">
         <x:v>6.93</x:v>
@@ -9153,7 +11538,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N8" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O8" s="31" t="str"/>
       <x:c r="P8" s="31" t="str"/>
@@ -9172,10 +11557,10 @@
         <x:v>modules/global manufacturing</x:v>
       </x:c>
       <x:c r="D9" s="30" t="n">
-        <x:v>22.662</x:v>
+        <x:v>22.49</x:v>
       </x:c>
       <x:c r="E9" s="30" t="n">
-        <x:v>1.2</x:v>
+        <x:v>1.18</x:v>
       </x:c>
       <x:c r="F9" s="30" t="n">
         <x:v>4.17</x:v>
@@ -9198,7 +11583,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N9" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O9" s="31" t="str"/>
       <x:c r="P9" s="31" t="str"/>
@@ -9217,17 +11602,17 @@
         <x:v>trackers</x:v>
       </x:c>
       <x:c r="D10" s="30" t="n">
-        <x:v>8.941</x:v>
+        <x:v>9.11</x:v>
       </x:c>
       <x:c r="E10" s="30" t="n">
-        <x:v>1.39</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="F10" s="30" t="n">
         <x:v>1.95</x:v>
       </x:c>
       <x:c r="G10" s="30" t="str"/>
       <x:c r="H10" s="30" t="n">
-        <x:v>12.22</x:v>
+        <x:v>12.37</x:v>
       </x:c>
       <x:c r="I10" s="30" t="n">
         <x:v>1.15</x:v>
@@ -9245,7 +11630,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N10" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O10" s="31" t="str"/>
       <x:c r="P10" s="31" t="str"/>
@@ -9264,19 +11649,19 @@
         <x:v>EBOS</x:v>
       </x:c>
       <x:c r="D11" s="30" t="n">
-        <x:v>12.15</x:v>
+        <x:v>12.069</x:v>
       </x:c>
       <x:c r="E11" s="30" t="n">
-        <x:v>2.05</x:v>
+        <x:v>2.01</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="G11" s="30" t="n">
-        <x:v>60.98</x:v>
+        <x:v>60.61</x:v>
       </x:c>
       <x:c r="H11" s="30" t="n">
-        <x:v>26.52</x:v>
+        <x:v>26.36</x:v>
       </x:c>
       <x:c r="I11" s="30" t="n">
         <x:v>3.8</x:v>
@@ -9294,7 +11679,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N11" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O11" s="31" t="str"/>
       <x:c r="P11" s="31" t="str"/>
@@ -9313,28 +11698,28 @@
         <x:v>trackers/software</x:v>
       </x:c>
       <x:c r="D12" s="30" t="n">
-        <x:v>133.116</x:v>
+        <x:v>133.015</x:v>
       </x:c>
       <x:c r="E12" s="30" t="n">
-        <x:v>20.12</x:v>
+        <x:v>20.01</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
-        <x:v>19.31</x:v>
+        <x:v>19.08</x:v>
       </x:c>
       <x:c r="G12" s="30" t="n">
-        <x:v>34.88</x:v>
+        <x:v>34.67</x:v>
       </x:c>
       <x:c r="H12" s="30" t="n">
-        <x:v>28.9</x:v>
+        <x:v>28.73</x:v>
       </x:c>
       <x:c r="I12" s="30" t="n">
-        <x:v>5.73</x:v>
+        <x:v>5.67</x:v>
       </x:c>
       <x:c r="J12" s="30" t="n">
-        <x:v>5.43</x:v>
+        <x:v>5.36</x:v>
       </x:c>
       <x:c r="K12" s="30" t="n">
-        <x:v>26.16</x:v>
+        <x:v>25.85</x:v>
       </x:c>
       <x:c r="L12" s="30" t="str">
         <x:v>S12</x:v>
@@ -9343,7 +11728,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N12" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O12" s="31" t="str"/>
       <x:c r="P12" s="31" t="str"/>
@@ -9362,19 +11747,19 @@
         <x:v>residential solar/service</x:v>
       </x:c>
       <x:c r="D13" s="30" t="n">
-        <x:v>15.24</x:v>
+        <x:v>15.36</x:v>
       </x:c>
       <x:c r="E13" s="30" t="n">
-        <x:v>3.65</x:v>
+        <x:v>3.66</x:v>
       </x:c>
       <x:c r="F13" s="30" t="n">
         <x:v>17.89</x:v>
       </x:c>
       <x:c r="G13" s="30" t="n">
-        <x:v>7.23</x:v>
+        <x:v>7.25</x:v>
       </x:c>
       <x:c r="H13" s="30" t="n">
-        <x:v>26.49</x:v>
+        <x:v>26.56</x:v>
       </x:c>
       <x:c r="I13" s="30" t="n">
         <x:v>1.16</x:v>
@@ -9392,7 +11777,7 @@
         <x:v>S11</x:v>
       </x:c>
       <x:c r="N13" s="30" t="str">
-        <x:v>Secondary market data snapshot; FSLR valuation cross-checks also use company filings and guidance.</x:v>
+        <x:v>Directional peer only: business model, margin structure, policy exposure and balance sheet differ from FSLR.</x:v>
       </x:c>
       <x:c r="O13" s="31" t="str"/>
       <x:c r="P13" s="31" t="str"/>
@@ -11460,7 +13845,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca8cd38509f4d5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d34fcc4e81d4a63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13979,9 +16364,9 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R841eba6ed14b4da6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R744bdde95e6e4944"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abccec0cd3b44d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raecac96a8c5a4592"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14252,28 +16637,28 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="str">
-        <x:v>Ongoing</x:v>
+        <x:v>2026-2029</x:v>
       </x:c>
       <x:c r="B10" s="20" t="str">
-        <x:v>Balance sheet</x:v>
+        <x:v>Execution / Demand</x:v>
       </x:c>
       <x:c r="C10" s="20" t="str">
-        <x:v>$1.5bn revolver and net cash</x:v>
+        <x:v>Backlog conversion and ASP durability</x:v>
       </x:c>
       <x:c r="D10" s="20" t="str">
-        <x:v>Strong liquidity</x:v>
+        <x:v>Core valuation driver</x:v>
       </x:c>
       <x:c r="E10" s="20" t="str">
-        <x:v>Net cash reduces downside and funds capacity; working capital swings can still move quarterly FCF.</x:v>
+        <x:v>Large backlog supports revenue visibility, but cancellations, delivery delays and lower new ASPs could weaken the 2027-2029 revenue bridge.</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
-        <x:v>Net cash, revolver draw, operating cash flow and capex.</x:v>
+        <x:v>Net bookings GW, backlog ASP, cancellations, delivery schedule, customer concentration.</x:v>
       </x:c>
       <x:c r="G10" s="20" t="str">
-        <x:v>Low/Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H10" s="20" t="str">
-        <x:v>S1;S2;S13</x:v>
+        <x:v>S1;S3;S4</x:v>
       </x:c>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
@@ -14283,14 +16668,30 @@
       <x:c r="N10" s="2"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="2"/>
-      <x:c r="C11" s="2"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-      <x:c r="G11" s="2"/>
-      <x:c r="H11" s="2"/>
+      <x:c r="A11" s="20" t="str">
+        <x:v>Ongoing</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>Balance sheet</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>$1.5bn revolver and net cash</x:v>
+      </x:c>
+      <x:c r="D11" s="20" t="str">
+        <x:v>Strong liquidity</x:v>
+      </x:c>
+      <x:c r="E11" s="20" t="str">
+        <x:v>Net cash reduces downside and funds capacity; working capital swings can still move quarterly FCF.</x:v>
+      </x:c>
+      <x:c r="F11" s="20" t="str">
+        <x:v>Net cash, revolver draw, operating cash flow and capex.</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>Low/Medium</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="str">
+        <x:v>S1;S2;S13</x:v>
+      </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -16369,7 +18770,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83dfd2ea077e4658"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R384fcd41ec374863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16476,19 +18877,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="20" t="str">
-        <x:v>FSLR 现在贵不贵？</x:v>
+        <x:v>Is FSLR fairly valued, overvalued, or still underappreciated given 2026 EBITDA power and policy-adjusted risk?</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>当前股价已接近基本情景，继续上行要靠 earnings power 抬升或估值倍数扩张。</x:v>
+        <x:v>当前估值已不便宜，但公司质量、45X、backlog 和净现金使 $290-$310 区间的风险收益仍偏正。</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>FY2026 EBITDA midpoint vs actual run-rate; EV/FY2026 EBITDA; TTM EPS; net cash.</x:v>
+        <x:v>FY2026 EBITDA run-rate, EV/FY2026 EBITDA, TTM P/E, net cash, policy-adjusted multiple.</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
-        <x:v>EV/FY2026 EBITDA &lt;9x 且 backlog ASP 稳定更适合分批；&gt;11-12x 需要明确政策/订单催化。</x:v>
+        <x:v>$290-$310 主动建仓；$260-$280 且 thesis intact 加仓；$360-$380 无经营上修则减仓；跌破 $250-$255 且出现 thesis break 则认错。</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>约 10.8x EV/FY2026 EBITDA midpoint；接近基本情景。</x:v>
+        <x:v>At ~11.0x FY2026 EBITDA and ~19.0x TTM P/E, FSLR is not deep value, but current-price risk/reward supports active building with explicit stop/reassessment triggers.</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
         <x:v>S1;S3;S11;S12</x:v>
@@ -16507,16 +18908,16 @@
         <x:v>backlog 是护城河还是峰值订单？</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
-        <x:v>47.9GW/$14.4bn 说明可见度强，但股票看的是新增订单价格和交付质量。</x:v>
+        <x:v>47.9GW/$14.4bn 说明可见度强，但股票看的是新增订单价格、取消风险和交付质量。</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>Net bookings GW, backlog value, backlog ASP, cancellations, delivery years.</x:v>
+        <x:v>Net bookings GW, new bookings ASP, backlog value, backlog ASP, cancellations, delivery years.</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
         <x:v>新增 bookings ASP 接近或高于 $0.30/W，且 2027-2029 交付不断档。</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>Q1 后 backlog ASP 约 $0.30/W；YTD bookings 3.7GW。</x:v>
+        <x:v>Q1 后 backlog ASP 约 $0.30/W；YTD bookings 3.7GW；下一步必须验证新增订单 ASP。</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>S1;S3</x:v>
@@ -16538,13 +18939,13 @@
         <x:v>45X 是 margin 和现金流的重要变量，政策折现率决定估值倍数。</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>45X recognized, cash realization, IRS/Treasury rules, PFE/FEOC restrictions.</x:v>
+        <x:v>45X recognized in gross profit, cash realization, tax-line treatment, IRS/Treasury rules, PFE/FEOC restrictions.</x:v>
       </x:c>
       <x:c r="D7" s="20" t="str">
         <x:v>规则稳定且公司披露现金化路径清晰，可降低市场折价。</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>FY2026 guide embeds about $2.145bn 45X credit；政策敏感度高。</x:v>
+        <x:v>FY2026 guide embeds about $2.145bn 45X credit；必须单独验证 cash realization，不能只看 EBITDA。</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>S3;S6;S7</x:v>
@@ -16594,13 +18995,13 @@
         <x:v>增长股要从 capex 周期切到 FCF 周期才更容易重估。</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>Production GW, sold GW, capex, OCF, inventory, warranty, efficiency.</x:v>
+        <x:v>Production GW, sold GW, capex, OCF, inventory, warranty, efficiency, OCF-capex conversion.</x:v>
       </x:c>
       <x:c r="D9" s="20" t="str">
         <x:v>OCF &gt; capex 的季度持续出现，同时产能利用率上行。</x:v>
       </x:c>
       <x:c r="E9" s="20" t="str">
-        <x:v>2025 OCF $2.06bn，capex $0.87bn；Q1 2026 OCF 为负，仍有季节性和营运资本波动。</x:v>
+        <x:v>2025 OCF $2.06bn，capex $0.87bn；Q1 2026 OCF -$214.9mn，需跟踪 Q2/Q3 是否恢复。</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>S2;S3;S4</x:v>
@@ -18717,7 +21118,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bc14d2f1ebd4fa7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R728e45de02ba4c8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18726,11 +21127,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16.25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16.25" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="53.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="45" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="16.25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16.25" hidden="0" customWidth="1"/>
@@ -18744,7 +21145,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Sources</x:v>
+        <x:v>Action Framework</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -18762,7 +21163,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>一手来源优先；每个数据表均通过 source_id 映射。</x:v>
+        <x:v>明确偏买、加仓、减仓和认错条件；价格带必须和经营触发器一起看。</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -18796,29 +21197,25 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="19" t="str">
+        <x:v>action</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>price_zone</x:v>
+      </x:c>
+      <x:c r="C4" s="19" t="str">
+        <x:v>position_action</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>operating_triggers</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>risk_control</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
         <x:v>source_id</x:v>
       </x:c>
-      <x:c r="B4" s="19" t="str">
-        <x:v>title</x:v>
-      </x:c>
-      <x:c r="C4" s="19" t="str">
-        <x:v>publisher</x:v>
-      </x:c>
-      <x:c r="D4" s="19" t="str">
-        <x:v>date</x:v>
-      </x:c>
-      <x:c r="E4" s="19" t="str">
-        <x:v>url</x:v>
-      </x:c>
-      <x:c r="F4" s="19" t="str">
-        <x:v>source_type</x:v>
-      </x:c>
-      <x:c r="G4" s="19" t="str">
-        <x:v>used_for</x:v>
-      </x:c>
-      <x:c r="H4" s="19" t="str">
-        <x:v>quality</x:v>
-      </x:c>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
       <x:c r="I4" s="2"/>
       <x:c r="J4" s="2"/>
       <x:c r="K4" s="2"/>
@@ -18828,29 +21225,25 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="20" t="str">
-        <x:v>S1</x:v>
+        <x:v>主动建仓</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>First Solar Q1 2026 earnings release, furnished as SEC 8-K Exhibit 99.1</x:v>
+        <x:v>$290-$310</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>First Solar / SEC</x:v>
+        <x:v>建立 40%-60% 目标仓位</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
-        <x:v>2026-04-30</x:v>
+        <x:v>无 45X、backlog、OCF 或 FY2026 guide 的 thesis break</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000108/ex991pressreleaseq1-2026.htm</x:v>
+        <x:v>不是一把梭；后续用经营触发器决定补仓或减仓</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
-        <x:v>company filing</x:v>
-      </x:c>
-      <x:c r="G5" s="20" t="str">
-        <x:v>Q1 revenue, EPS, EBITDA, cash, debt, guidance, backlog</x:v>
-      </x:c>
-      <x:c r="H5" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S11;S12</x:v>
+      </x:c>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="2"/>
       <x:c r="K5" s="2"/>
@@ -18860,29 +21253,25 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="str">
-        <x:v>S2</x:v>
+        <x:v>回撤加仓</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
-        <x:v>First Solar Form 10-Q for quarter ended March 31, 2026</x:v>
+        <x:v>$260-$280</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>SEC</x:v>
+        <x:v>补到 70%-90% 目标仓位</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
-        <x:v>2026-04-30</x:v>
+        <x:v>backlog ASP 稳定、无重大取消/延迟，45X 现金化路径未恶化</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000109/fslr-20260331.htm</x:v>
+        <x:v>若回撤来自政策或订单实质恶化，不加仓</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
-        <x:v>SEC filing</x:v>
-      </x:c>
-      <x:c r="G6" s="20" t="str">
-        <x:v>Q1 financial statements, capacity and policy-risk wording</x:v>
-      </x:c>
-      <x:c r="H6" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S6;S7</x:v>
+      </x:c>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
@@ -18892,29 +21281,25 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="20" t="str">
-        <x:v>S3</x:v>
+        <x:v>确认加仓</x:v>
       </x:c>
       <x:c r="B7" s="20" t="str">
-        <x:v>First Solar Q1 2026 earnings presentation</x:v>
+        <x:v>$310-$330</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>First Solar</x:v>
+        <x:v>最多补到满仓</x:v>
       </x:c>
       <x:c r="D7" s="20" t="str">
-        <x:v>2026-04-30</x:v>
+        <x:v>新增 bookings ASP 接近/高于 $0.30/W；45X cash realization 清晰；OCF-capex 转正；2027-2029 收入桥更清楚，至少满足两项</x:v>
       </x:c>
       <x:c r="E7" s="20" t="str">
-        <x:v>https://s202.q4cdn.com/499595574/files/doc_financials/2026/q1/Q1-26-Earnings-Presentation-vf-Secured.pdf</x:v>
+        <x:v>只为经营确认加仓，不为单日政策新闻追价</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
-        <x:v>company presentation</x:v>
-      </x:c>
-      <x:c r="G7" s="20" t="str">
-        <x:v>bookings, backlog, guide ranges, capacity, 45X guide, shipment and sales volume</x:v>
-      </x:c>
-      <x:c r="H7" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S6;S7;S8;S9</x:v>
+      </x:c>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
@@ -18924,29 +21309,25 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="str">
-        <x:v>S4</x:v>
+        <x:v>持有观察</x:v>
       </x:c>
       <x:c r="B8" s="20" t="str">
-        <x:v>First Solar Form 10-K for fiscal year 2025</x:v>
+        <x:v>$330-$360</x:v>
       </x:c>
       <x:c r="C8" s="20" t="str">
-        <x:v>SEC</x:v>
+        <x:v>持有，不主动扩仓</x:v>
       </x:c>
       <x:c r="D8" s="20" t="str">
-        <x:v>2026-02-24</x:v>
+        <x:v>FY2026 EBITDA run-rate、毛利率和 backlog conversion 与模型一致</x:v>
       </x:c>
       <x:c r="E8" s="20" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000021/fslr-20251231.htm</x:v>
+        <x:v>若估值先涨而经营未上修，准备减仓</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
-        <x:v>SEC filing</x:v>
-      </x:c>
-      <x:c r="G8" s="20" t="str">
-        <x:v>FY2023-FY2025 financials, cash flow, operating drivers</x:v>
-      </x:c>
-      <x:c r="H8" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S12</x:v>
+      </x:c>
+      <x:c r="G8" s="2"/>
+      <x:c r="H8" s="2"/>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
@@ -18956,29 +21337,25 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="20" t="str">
-        <x:v>S5</x:v>
+        <x:v>减仓</x:v>
       </x:c>
       <x:c r="B9" s="20" t="str">
-        <x:v>First Solar Q4/FY2025 earnings release, furnished as SEC 8-K Exhibit 99.1</x:v>
+        <x:v>$360-$380</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>First Solar / SEC</x:v>
+        <x:v>降低 20%-40% 仓位</x:v>
       </x:c>
       <x:c r="D9" s="20" t="str">
-        <x:v>2026-02-24</x:v>
+        <x:v>股价接近 bull case，但没有 EBITDA、backlog ASP 或 45X 确定性上修；或 EV/FY2026 EBITDA 高于约 13x</x:v>
       </x:c>
       <x:c r="E9" s="20" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000020/ex991pressreleaseq4-2025fi.htm</x:v>
+        <x:v>保留核心仓位等待下一轮数据，不把 bull case 当 base case</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
-        <x:v>company filing</x:v>
-      </x:c>
-      <x:c r="G9" s="20" t="str">
-        <x:v>FY2025 results, 2026 guide baseline, year-end backlog</x:v>
-      </x:c>
-      <x:c r="H9" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S12</x:v>
+      </x:c>
+      <x:c r="G9" s="2"/>
+      <x:c r="H9" s="2"/>
       <x:c r="I9" s="2"/>
       <x:c r="J9" s="2"/>
       <x:c r="K9" s="2"/>
@@ -18988,29 +21365,25 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="str">
-        <x:v>S6</x:v>
+        <x:v>认错/止损</x:v>
       </x:c>
       <x:c r="B10" s="20" t="str">
-        <x:v>IRS final regulations for Section 45X advanced manufacturing production credit</x:v>
+        <x:v>&lt;$250-$255 或经营触发器失效</x:v>
       </x:c>
       <x:c r="C10" s="20" t="str">
-        <x:v>IRS</x:v>
+        <x:v>减至小仓或退出并重做模型</x:v>
       </x:c>
       <x:c r="D10" s="20" t="str">
-        <x:v>2024-12-16</x:v>
+        <x:v>FY2026 EBITDA run-rate/guide 低于约 $2.5bn；新增 bookings ASP &lt; $0.27/W；重大取消/延迟；45X 现金化受阻；OCF-capex 连续两个季度不恢复；2027-2029 收入桥断档</x:v>
       </x:c>
       <x:c r="E10" s="20" t="str">
-        <x:v>https://www.irs.gov/irb/2024-51_IRB/index.html</x:v>
+        <x:v>价格跌破区间必须结合 thesis break；经营触发器失效时不等价格确认</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
-        <x:v>official policy</x:v>
-      </x:c>
-      <x:c r="G10" s="20" t="str">
-        <x:v>45X credit qualification and solar module components</x:v>
-      </x:c>
-      <x:c r="H10" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+        <x:v>S1;S3;S6;S7;S11;S12</x:v>
+      </x:c>
+      <x:c r="G10" s="2"/>
+      <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
       <x:c r="K10" s="2"/>
@@ -19019,30 +21392,14 @@
       <x:c r="N10" s="2"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="20" t="str">
-        <x:v>S7</x:v>
-      </x:c>
-      <x:c r="B11" s="20" t="str">
-        <x:v>IRS clean energy provisions of the One Big Beautiful Bill Act</x:v>
-      </x:c>
-      <x:c r="C11" s="20" t="str">
-        <x:v>IRS</x:v>
-      </x:c>
-      <x:c r="D11" s="20" t="str">
-        <x:v>2025-08-28</x:v>
-      </x:c>
-      <x:c r="E11" s="20" t="str">
-        <x:v>https://www.irs.gov/credits-deductions/one-big-beautiful-bill-act-provisions-for-individuals-and-businesses</x:v>
-      </x:c>
-      <x:c r="F11" s="20" t="str">
-        <x:v>official policy</x:v>
-      </x:c>
-      <x:c r="G11" s="20" t="str">
-        <x:v>post-OBBBA clean-energy-credit constraints and FEOC/PFE monitor</x:v>
-      </x:c>
-      <x:c r="H11" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A11" s="2"/>
+      <x:c r="B11" s="2"/>
+      <x:c r="C11" s="2"/>
+      <x:c r="D11" s="2"/>
+      <x:c r="E11" s="2"/>
+      <x:c r="F11" s="2"/>
+      <x:c r="G11" s="2"/>
+      <x:c r="H11" s="2"/>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -19051,30 +21408,14 @@
       <x:c r="N11" s="2"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="20" t="str">
-        <x:v>S8</x:v>
-      </x:c>
-      <x:c r="B12" s="20" t="str">
-        <x:v>Commerce final determinations in solar cells from Cambodia, Malaysia, Thailand and Vietnam</x:v>
-      </x:c>
-      <x:c r="C12" s="20" t="str">
-        <x:v>U.S. Department of Commerce</x:v>
-      </x:c>
-      <x:c r="D12" s="20" t="str">
-        <x:v>2025-04-21</x:v>
-      </x:c>
-      <x:c r="E12" s="20" t="str">
-        <x:v>https://www.trade.gov/press-release/us-department-commerce-announces-final-determinations-antidumping-and-countervailing</x:v>
-      </x:c>
-      <x:c r="F12" s="20" t="str">
-        <x:v>official trade policy</x:v>
-      </x:c>
-      <x:c r="G12" s="20" t="str">
-        <x:v>AD/CVD tariff risk and domestic supply-demand context</x:v>
-      </x:c>
-      <x:c r="H12" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A12" s="2"/>
+      <x:c r="B12" s="2"/>
+      <x:c r="C12" s="2"/>
+      <x:c r="D12" s="2"/>
+      <x:c r="E12" s="2"/>
+      <x:c r="F12" s="2"/>
+      <x:c r="G12" s="2"/>
+      <x:c r="H12" s="2"/>
       <x:c r="I12" s="2"/>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -19083,30 +21424,14 @@
       <x:c r="N12" s="2"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="20" t="str">
-        <x:v>S9</x:v>
-      </x:c>
-      <x:c r="B13" s="20" t="str">
-        <x:v>BIS Section 232 investigations page</x:v>
-      </x:c>
-      <x:c r="C13" s="20" t="str">
-        <x:v>U.S. Bureau of Industry and Security</x:v>
-      </x:c>
-      <x:c r="D13" s="20" t="str">
-        <x:v>2026-05-28</x:v>
-      </x:c>
-      <x:c r="E13" s="20" t="str">
-        <x:v>https://www.bis.doc.gov/index.php/232</x:v>
-      </x:c>
-      <x:c r="F13" s="20" t="str">
-        <x:v>official trade policy</x:v>
-      </x:c>
-      <x:c r="G13" s="20" t="str">
-        <x:v>Section 232 polysilicon/derivatives status tracker</x:v>
-      </x:c>
-      <x:c r="H13" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A13" s="2"/>
+      <x:c r="B13" s="2"/>
+      <x:c r="C13" s="2"/>
+      <x:c r="D13" s="2"/>
+      <x:c r="E13" s="2"/>
+      <x:c r="F13" s="2"/>
+      <x:c r="G13" s="2"/>
+      <x:c r="H13" s="2"/>
       <x:c r="I13" s="2"/>
       <x:c r="J13" s="2"/>
       <x:c r="K13" s="2"/>
@@ -19115,30 +21440,14 @@
       <x:c r="N13" s="2"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="20" t="str">
-        <x:v>S10</x:v>
-      </x:c>
-      <x:c r="B14" s="20" t="str">
-        <x:v>USITC Section 337 TOPCon solar cells investigation docket</x:v>
-      </x:c>
-      <x:c r="C14" s="20" t="str">
-        <x:v>U.S. International Trade Commission</x:v>
-      </x:c>
-      <x:c r="D14" s="20" t="str">
-        <x:v>2026-03-26</x:v>
-      </x:c>
-      <x:c r="E14" s="20" t="str">
-        <x:v>https://www.usitc.gov/press_room/news_release/2026/er0326_67276.htm</x:v>
-      </x:c>
-      <x:c r="F14" s="20" t="str">
-        <x:v>official litigation/regulatory</x:v>
-      </x:c>
-      <x:c r="G14" s="20" t="str">
-        <x:v>patent/import catalyst and policy risk tracker</x:v>
-      </x:c>
-      <x:c r="H14" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="2"/>
+      <x:c r="C14" s="2"/>
+      <x:c r="D14" s="2"/>
+      <x:c r="E14" s="2"/>
+      <x:c r="F14" s="2"/>
+      <x:c r="G14" s="2"/>
+      <x:c r="H14" s="2"/>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="2"/>
       <x:c r="K14" s="2"/>
@@ -19147,30 +21456,14 @@
       <x:c r="N14" s="2"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="20" t="str">
-        <x:v>S11</x:v>
-      </x:c>
-      <x:c r="B15" s="20" t="str">
-        <x:v>Yahoo Finance chart API and quote pages</x:v>
-      </x:c>
-      <x:c r="C15" s="20" t="str">
-        <x:v>Yahoo Finance</x:v>
-      </x:c>
-      <x:c r="D15" s="20" t="str">
-        <x:v>2026-05-28</x:v>
-      </x:c>
-      <x:c r="E15" s="20" t="str">
-        <x:v>https://finance.yahoo.com/quote/FSLR</x:v>
-      </x:c>
-      <x:c r="F15" s="20" t="str">
-        <x:v>market data</x:v>
-      </x:c>
-      <x:c r="G15" s="20" t="str">
-        <x:v>current quote and event-window close-to-close market reactions</x:v>
-      </x:c>
-      <x:c r="H15" s="20" t="str">
-        <x:v>market data</x:v>
-      </x:c>
+      <x:c r="A15" s="2"/>
+      <x:c r="B15" s="2"/>
+      <x:c r="C15" s="2"/>
+      <x:c r="D15" s="2"/>
+      <x:c r="E15" s="2"/>
+      <x:c r="F15" s="2"/>
+      <x:c r="G15" s="2"/>
+      <x:c r="H15" s="2"/>
       <x:c r="I15" s="2"/>
       <x:c r="J15" s="2"/>
       <x:c r="K15" s="2"/>
@@ -19179,30 +21472,14 @@
       <x:c r="N15" s="2"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="20" t="str">
-        <x:v>S12</x:v>
-      </x:c>
-      <x:c r="B16" s="20" t="str">
-        <x:v>StockAnalysis valuation statistics pages</x:v>
-      </x:c>
-      <x:c r="C16" s="20" t="str">
-        <x:v>StockAnalysis</x:v>
-      </x:c>
-      <x:c r="D16" s="20" t="str">
-        <x:v>2026-05-28</x:v>
-      </x:c>
-      <x:c r="E16" s="20" t="str">
-        <x:v>https://stockanalysis.com/stocks/fslr/statistics/</x:v>
-      </x:c>
-      <x:c r="F16" s="20" t="str">
-        <x:v>secondary market data</x:v>
-      </x:c>
-      <x:c r="G16" s="20" t="str">
-        <x:v>market cap, EV, peer valuation snapshots</x:v>
-      </x:c>
-      <x:c r="H16" s="20" t="str">
-        <x:v>secondary</x:v>
-      </x:c>
+      <x:c r="A16" s="2"/>
+      <x:c r="B16" s="2"/>
+      <x:c r="C16" s="2"/>
+      <x:c r="D16" s="2"/>
+      <x:c r="E16" s="2"/>
+      <x:c r="F16" s="2"/>
+      <x:c r="G16" s="2"/>
+      <x:c r="H16" s="2"/>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
       <x:c r="K16" s="2"/>
@@ -19211,30 +21488,14 @@
       <x:c r="N16" s="2"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="20" t="str">
-        <x:v>S13</x:v>
-      </x:c>
-      <x:c r="B17" s="20" t="str">
-        <x:v>First Solar 8-K: $1.5B senior unsecured revolving credit facility</x:v>
-      </x:c>
-      <x:c r="C17" s="20" t="str">
-        <x:v>SEC</x:v>
-      </x:c>
-      <x:c r="D17" s="20" t="str">
-        <x:v>2026-02-19</x:v>
-      </x:c>
-      <x:c r="E17" s="20" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000016/fslr-20260213.htm</x:v>
-      </x:c>
-      <x:c r="F17" s="20" t="str">
-        <x:v>SEC filing</x:v>
-      </x:c>
-      <x:c r="G17" s="20" t="str">
-        <x:v>liquidity and balance-sheet catalyst</x:v>
-      </x:c>
-      <x:c r="H17" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A17" s="2"/>
+      <x:c r="B17" s="2"/>
+      <x:c r="C17" s="2"/>
+      <x:c r="D17" s="2"/>
+      <x:c r="E17" s="2"/>
+      <x:c r="F17" s="2"/>
+      <x:c r="G17" s="2"/>
+      <x:c r="H17" s="2"/>
       <x:c r="I17" s="2"/>
       <x:c r="J17" s="2"/>
       <x:c r="K17" s="2"/>
@@ -19243,30 +21504,14 @@
       <x:c r="N17" s="2"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="20" t="str">
-        <x:v>S14</x:v>
-      </x:c>
-      <x:c r="B18" s="20" t="str">
-        <x:v>USITC sunset reviews: crystalline silicon photovoltaic cells and modules from China and Taiwan</x:v>
-      </x:c>
-      <x:c r="C18" s="20" t="str">
-        <x:v>U.S. International Trade Commission</x:v>
-      </x:c>
-      <x:c r="D18" s="20" t="str">
-        <x:v>2026-05-27</x:v>
-      </x:c>
-      <x:c r="E18" s="20" t="str">
-        <x:v>https://www.usitc.gov/press_room/news_release/2026/er0527_67584.htm</x:v>
-      </x:c>
-      <x:c r="F18" s="20" t="str">
-        <x:v>official trade policy</x:v>
-      </x:c>
-      <x:c r="G18" s="20" t="str">
-        <x:v>tariff continuation catalyst</x:v>
-      </x:c>
-      <x:c r="H18" s="20" t="str">
-        <x:v>primary</x:v>
-      </x:c>
+      <x:c r="A18" s="2"/>
+      <x:c r="B18" s="2"/>
+      <x:c r="C18" s="2"/>
+      <x:c r="D18" s="2"/>
+      <x:c r="E18" s="2"/>
+      <x:c r="F18" s="2"/>
+      <x:c r="G18" s="2"/>
+      <x:c r="H18" s="2"/>
       <x:c r="I18" s="2"/>
       <x:c r="J18" s="2"/>
       <x:c r="K18" s="2"/>
@@ -21233,7 +23478,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb32f7c2a01dc423d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70186a70472b4197"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21260,7 +23505,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Sources</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -21278,7 +23523,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Sanity checks：公式、来源、口径和空值。</x:v>
+        <x:v>一手来源优先；每个数据表均通过 source_id 映射。</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -21311,22 +23556,30 @@
       <x:c r="N3" s="2"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="7" t="str">
-        <x:v>Check</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="str">
-        <x:v>Formula result</x:v>
-      </x:c>
-      <x:c r="C4" s="7" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="D4" s="7" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="E4" s="2"/>
-      <x:c r="F4" s="2"/>
-      <x:c r="G4" s="2"/>
-      <x:c r="H4" s="2"/>
+      <x:c r="A4" s="19" t="str">
+        <x:v>source_id</x:v>
+      </x:c>
+      <x:c r="B4" s="19" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="C4" s="19" t="str">
+        <x:v>publisher</x:v>
+      </x:c>
+      <x:c r="D4" s="19" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>url</x:v>
+      </x:c>
+      <x:c r="F4" s="19" t="str">
+        <x:v>source_type</x:v>
+      </x:c>
+      <x:c r="G4" s="19" t="str">
+        <x:v>used_for</x:v>
+      </x:c>
+      <x:c r="H4" s="19" t="str">
+        <x:v>quality</x:v>
+      </x:c>
       <x:c r="I4" s="2"/>
       <x:c r="J4" s="2"/>
       <x:c r="K4" s="2"/>
@@ -21335,24 +23588,30 @@
       <x:c r="N4" s="2"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="2" t="str">
-        <x:v>Q1 revenue YoY ties to release</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="b">
-        <x:f>ABS(('Financials KPIs'!H5/'Financials KPIs'!G5-1)-0.236)&lt;0.02</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="2" t="str">
-        <x:f>IF(B5,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D5" s="2" t="str">
-        <x:v>Expected about 24%</x:v>
-      </x:c>
-      <x:c r="E5" s="2"/>
-      <x:c r="F5" s="2"/>
-      <x:c r="G5" s="2"/>
-      <x:c r="H5" s="2"/>
+      <x:c r="A5" s="20" t="str">
+        <x:v>S1</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="str">
+        <x:v>First Solar Q1 2026 earnings release, furnished as SEC 8-K Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="str">
+        <x:v>First Solar / SEC</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="str">
+        <x:v>2026-04-30</x:v>
+      </x:c>
+      <x:c r="E5" s="20" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000108/ex991pressreleaseq1-2026.htm</x:v>
+      </x:c>
+      <x:c r="F5" s="20" t="str">
+        <x:v>company filing</x:v>
+      </x:c>
+      <x:c r="G5" s="20" t="str">
+        <x:v>Q1 revenue, EPS, EBITDA, cash, debt, guidance, backlog</x:v>
+      </x:c>
+      <x:c r="H5" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="2"/>
       <x:c r="K5" s="2"/>
@@ -21361,24 +23620,30 @@
       <x:c r="N5" s="2"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="2" t="str">
-        <x:v>Gross margin recalculates from Q1 revenue/gross profit</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="b">
-        <x:f>ABS(('Financials KPIs'!H6/'Financials KPIs'!H5*100)-'Financials KPIs'!H7)&lt;0.1</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="2" t="str">
-        <x:f>IF(B6,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D6" s="2" t="str">
-        <x:v>Q1 2026 gross margin should be about 46.6%</x:v>
-      </x:c>
-      <x:c r="E6" s="2"/>
-      <x:c r="F6" s="2"/>
-      <x:c r="G6" s="2"/>
-      <x:c r="H6" s="2"/>
+      <x:c r="A6" s="20" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="str">
+        <x:v>First Solar Form 10-Q for quarter ended March 31, 2026</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="str">
+        <x:v>2026-04-30</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000109/fslr-20260331.htm</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
+        <x:v>SEC filing</x:v>
+      </x:c>
+      <x:c r="G6" s="20" t="str">
+        <x:v>Q1 financial statements, capacity and policy-risk wording</x:v>
+      </x:c>
+      <x:c r="H6" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I6" s="2"/>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
@@ -21387,24 +23652,30 @@
       <x:c r="N6" s="2"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="2" t="str">
-        <x:v>EV equals market cap minus net cash</x:v>
-      </x:c>
-      <x:c r="B7" s="2" t="b">
-        <x:f>ABS(Valuation!B9-(Valuation!B7-Valuation!B8))&lt;0.01</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="2" t="str">
-        <x:f>IF(B7,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D7" s="2" t="str">
-        <x:v>Valuation formula cross-check</x:v>
-      </x:c>
-      <x:c r="E7" s="2"/>
-      <x:c r="F7" s="2"/>
-      <x:c r="G7" s="2"/>
-      <x:c r="H7" s="2"/>
+      <x:c r="A7" s="20" t="str">
+        <x:v>S3</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="str">
+        <x:v>First Solar Q1 2026 earnings presentation</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="str">
+        <x:v>First Solar</x:v>
+      </x:c>
+      <x:c r="D7" s="20" t="str">
+        <x:v>2026-04-30</x:v>
+      </x:c>
+      <x:c r="E7" s="20" t="str">
+        <x:v>https://s202.q4cdn.com/499595574/files/doc_financials/2026/q1/Q1-26-Earnings-Presentation-vf-Secured.pdf</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
+        <x:v>company presentation</x:v>
+      </x:c>
+      <x:c r="G7" s="20" t="str">
+        <x:v>bookings, backlog, guide ranges, capacity, 45X guide, shipment and sales volume</x:v>
+      </x:c>
+      <x:c r="H7" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
@@ -21413,24 +23684,30 @@
       <x:c r="N7" s="2"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="2" t="str">
-        <x:v>Backlog ASP equals backlog value / backlog GW</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="b">
-        <x:f>ABS(Valuation!B18-(Valuation!B17/Valuation!B16))&lt;0.001</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C8" s="2" t="str">
-        <x:f>IF(B8,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D8" s="2" t="str">
-        <x:v>Backlog value is USD bn; GW maps to $/W</x:v>
-      </x:c>
-      <x:c r="E8" s="2"/>
-      <x:c r="F8" s="2"/>
-      <x:c r="G8" s="2"/>
-      <x:c r="H8" s="2"/>
+      <x:c r="A8" s="20" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="str">
+        <x:v>First Solar Form 10-K for fiscal year 2025</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D8" s="20" t="str">
+        <x:v>2026-02-24</x:v>
+      </x:c>
+      <x:c r="E8" s="20" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000021/fslr-20251231.htm</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
+        <x:v>SEC filing</x:v>
+      </x:c>
+      <x:c r="G8" s="20" t="str">
+        <x:v>FY2023-FY2025 financials, cash flow, operating drivers</x:v>
+      </x:c>
+      <x:c r="H8" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
@@ -21439,24 +23716,30 @@
       <x:c r="N8" s="2"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="2" t="str">
-        <x:v>Source count &gt;= 12</x:v>
-      </x:c>
-      <x:c r="B9" s="2" t="b">
-        <x:f>COUNTA(Sources!A5:A50)&gt;=12</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="2" t="str">
-        <x:f>IF(B9,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D9" s="2" t="str">
-        <x:v>Coverage and citation sanity check</x:v>
-      </x:c>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
-      <x:c r="G9" s="2"/>
-      <x:c r="H9" s="2"/>
+      <x:c r="A9" s="20" t="str">
+        <x:v>S5</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="str">
+        <x:v>First Solar Q4/FY2025 earnings release, furnished as SEC 8-K Exhibit 99.1</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str">
+        <x:v>First Solar / SEC</x:v>
+      </x:c>
+      <x:c r="D9" s="20" t="str">
+        <x:v>2026-02-24</x:v>
+      </x:c>
+      <x:c r="E9" s="20" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000020/ex991pressreleaseq4-2025fi.htm</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
+        <x:v>company filing</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>FY2025 results, 2026 guide baseline, year-end backlog</x:v>
+      </x:c>
+      <x:c r="H9" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I9" s="2"/>
       <x:c r="J9" s="2"/>
       <x:c r="K9" s="2"/>
@@ -21465,24 +23748,30 @@
       <x:c r="N9" s="2"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="2" t="str">
-        <x:v>Critical valuation inputs are nonblank</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="b">
-        <x:f>COUNTBLANK(Valuation!B5:B18)=0</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="2" t="str">
-        <x:f>IF(B10,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D10" s="2" t="str">
-        <x:v>Avoid silent blank-driven formulas</x:v>
-      </x:c>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
-      <x:c r="G10" s="2"/>
-      <x:c r="H10" s="2"/>
+      <x:c r="A10" s="20" t="str">
+        <x:v>S6</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>IRS final regulations for Section 45X advanced manufacturing production credit</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str">
+        <x:v>IRS</x:v>
+      </x:c>
+      <x:c r="D10" s="20" t="str">
+        <x:v>2024-12-16</x:v>
+      </x:c>
+      <x:c r="E10" s="20" t="str">
+        <x:v>https://www.irs.gov/irb/2024-51_IRB/index.html</x:v>
+      </x:c>
+      <x:c r="F10" s="20" t="str">
+        <x:v>official policy</x:v>
+      </x:c>
+      <x:c r="G10" s="20" t="str">
+        <x:v>45X credit qualification and solar module components</x:v>
+      </x:c>
+      <x:c r="H10" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I10" s="2"/>
       <x:c r="J10" s="2"/>
       <x:c r="K10" s="2"/>
@@ -21491,24 +23780,30 @@
       <x:c r="N10" s="2"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="2" t="str">
-        <x:v>Market reaction alpha formula ties</x:v>
-      </x:c>
-      <x:c r="B11" s="2" t="b">
-        <x:f>ABS('Market Reaction'!N5-('Market Reaction'!I5-'Market Reaction'!J5))&lt;0.01</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C11" s="2" t="str">
-        <x:f>IF(B11,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D11" s="2" t="str">
-        <x:v>alpha = FSLR return - TAN return</x:v>
-      </x:c>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-      <x:c r="G11" s="2"/>
-      <x:c r="H11" s="2"/>
+      <x:c r="A11" s="20" t="str">
+        <x:v>S7</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>IRS clean energy provisions of the One Big Beautiful Bill Act</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>IRS</x:v>
+      </x:c>
+      <x:c r="D11" s="20" t="str">
+        <x:v>2025-08-28</x:v>
+      </x:c>
+      <x:c r="E11" s="20" t="str">
+        <x:v>https://www.irs.gov/credits-deductions/one-big-beautiful-bill-act-provisions-for-individuals-and-businesses</x:v>
+      </x:c>
+      <x:c r="F11" s="20" t="str">
+        <x:v>official policy</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="str">
+        <x:v>post-OBBBA clean-energy-credit constraints and FEOC/PFE monitor</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I11" s="2"/>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -21517,24 +23812,30 @@
       <x:c r="N11" s="2"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="2" t="str">
-        <x:v>FY2026 EBITDA midpoint is $2.7bn</x:v>
-      </x:c>
-      <x:c r="B12" s="2" t="b">
-        <x:f>ABS(Valuation!B11-2.7)&lt;0.001</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="str">
-        <x:f>IF(B12,"OK","CHECK")</x:f>
-        <x:v>OK</x:v>
-      </x:c>
-      <x:c r="D12" s="2" t="str">
-        <x:v>From $2.6-$2.8bn guidance</x:v>
-      </x:c>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
-      <x:c r="G12" s="2"/>
-      <x:c r="H12" s="2"/>
+      <x:c r="A12" s="20" t="str">
+        <x:v>S8</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="str">
+        <x:v>Commerce final determinations in solar cells from Cambodia, Malaysia, Thailand and Vietnam</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="str">
+        <x:v>U.S. Department of Commerce</x:v>
+      </x:c>
+      <x:c r="D12" s="20" t="str">
+        <x:v>2025-04-21</x:v>
+      </x:c>
+      <x:c r="E12" s="20" t="str">
+        <x:v>https://www.trade.gov/press-release/us-department-commerce-announces-final-determinations-antidumping-and-countervailing</x:v>
+      </x:c>
+      <x:c r="F12" s="20" t="str">
+        <x:v>official trade policy</x:v>
+      </x:c>
+      <x:c r="G12" s="20" t="str">
+        <x:v>AD/CVD tariff risk and domestic supply-demand context</x:v>
+      </x:c>
+      <x:c r="H12" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I12" s="2"/>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -21543,14 +23844,30 @@
       <x:c r="N12" s="2"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="2"/>
-      <x:c r="B13" s="2"/>
-      <x:c r="C13" s="2"/>
-      <x:c r="D13" s="2"/>
-      <x:c r="E13" s="2"/>
-      <x:c r="F13" s="2"/>
-      <x:c r="G13" s="2"/>
-      <x:c r="H13" s="2"/>
+      <x:c r="A13" s="20" t="str">
+        <x:v>S9</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="str">
+        <x:v>BIS Section 232 investigations page</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="str">
+        <x:v>U.S. Bureau of Industry and Security</x:v>
+      </x:c>
+      <x:c r="D13" s="20" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="E13" s="20" t="str">
+        <x:v>https://www.bis.doc.gov/index.php/232</x:v>
+      </x:c>
+      <x:c r="F13" s="20" t="str">
+        <x:v>official trade policy</x:v>
+      </x:c>
+      <x:c r="G13" s="20" t="str">
+        <x:v>Section 232 polysilicon/derivatives status tracker</x:v>
+      </x:c>
+      <x:c r="H13" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I13" s="2"/>
       <x:c r="J13" s="2"/>
       <x:c r="K13" s="2"/>
@@ -21559,14 +23876,30 @@
       <x:c r="N13" s="2"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="2"/>
-      <x:c r="C14" s="2"/>
-      <x:c r="D14" s="2"/>
-      <x:c r="E14" s="2"/>
-      <x:c r="F14" s="2"/>
-      <x:c r="G14" s="2"/>
-      <x:c r="H14" s="2"/>
+      <x:c r="A14" s="20" t="str">
+        <x:v>S10</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="str">
+        <x:v>USITC Section 337 TOPCon solar cells investigation docket</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="str">
+        <x:v>U.S. International Trade Commission</x:v>
+      </x:c>
+      <x:c r="D14" s="20" t="str">
+        <x:v>2026-03-26</x:v>
+      </x:c>
+      <x:c r="E14" s="20" t="str">
+        <x:v>https://www.usitc.gov/press_room/news_release/2026/er0326_67276.htm</x:v>
+      </x:c>
+      <x:c r="F14" s="20" t="str">
+        <x:v>official litigation/regulatory</x:v>
+      </x:c>
+      <x:c r="G14" s="20" t="str">
+        <x:v>patent/import catalyst and policy risk tracker</x:v>
+      </x:c>
+      <x:c r="H14" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="2"/>
       <x:c r="K14" s="2"/>
@@ -21575,14 +23908,30 @@
       <x:c r="N14" s="2"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
-      <x:c r="F15" s="2"/>
-      <x:c r="G15" s="2"/>
-      <x:c r="H15" s="2"/>
+      <x:c r="A15" s="20" t="str">
+        <x:v>S11</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="str">
+        <x:v>Yahoo Finance chart API and quote pages</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="str">
+        <x:v>Yahoo Finance</x:v>
+      </x:c>
+      <x:c r="D15" s="20" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="E15" s="20" t="str">
+        <x:v>https://finance.yahoo.com/quote/FSLR</x:v>
+      </x:c>
+      <x:c r="F15" s="20" t="str">
+        <x:v>market data</x:v>
+      </x:c>
+      <x:c r="G15" s="20" t="str">
+        <x:v>current quote and event-window close-to-close market reactions</x:v>
+      </x:c>
+      <x:c r="H15" s="20" t="str">
+        <x:v>market data</x:v>
+      </x:c>
       <x:c r="I15" s="2"/>
       <x:c r="J15" s="2"/>
       <x:c r="K15" s="2"/>
@@ -21591,14 +23940,30 @@
       <x:c r="N15" s="2"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2"/>
+      <x:c r="A16" s="20" t="str">
+        <x:v>S12</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="str">
+        <x:v>StockAnalysis valuation statistics pages</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>StockAnalysis</x:v>
+      </x:c>
+      <x:c r="D16" s="20" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="E16" s="20" t="str">
+        <x:v>https://stockanalysis.com/stocks/fslr/statistics/</x:v>
+      </x:c>
+      <x:c r="F16" s="20" t="str">
+        <x:v>secondary market data</x:v>
+      </x:c>
+      <x:c r="G16" s="20" t="str">
+        <x:v>market cap, EV, peer valuation snapshots</x:v>
+      </x:c>
+      <x:c r="H16" s="20" t="str">
+        <x:v>secondary</x:v>
+      </x:c>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
       <x:c r="K16" s="2"/>
@@ -21607,14 +23972,30 @@
       <x:c r="N16" s="2"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
+      <x:c r="A17" s="20" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="str">
+        <x:v>First Solar 8-K: $1.5B senior unsecured revolving credit facility</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="str">
+        <x:v>SEC</x:v>
+      </x:c>
+      <x:c r="D17" s="20" t="str">
+        <x:v>2026-02-19</x:v>
+      </x:c>
+      <x:c r="E17" s="20" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1274494/000127449426000016/fslr-20260213.htm</x:v>
+      </x:c>
+      <x:c r="F17" s="20" t="str">
+        <x:v>SEC filing</x:v>
+      </x:c>
+      <x:c r="G17" s="20" t="str">
+        <x:v>liquidity and balance-sheet catalyst</x:v>
+      </x:c>
+      <x:c r="H17" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I17" s="2"/>
       <x:c r="J17" s="2"/>
       <x:c r="K17" s="2"/>
@@ -21623,14 +24004,30 @@
       <x:c r="N17" s="2"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
-      <x:c r="E18" s="2"/>
-      <x:c r="F18" s="2"/>
-      <x:c r="G18" s="2"/>
-      <x:c r="H18" s="2"/>
+      <x:c r="A18" s="20" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>USITC sunset reviews: crystalline silicon photovoltaic cells and modules from China and Taiwan</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>U.S. International Trade Commission</x:v>
+      </x:c>
+      <x:c r="D18" s="20" t="str">
+        <x:v>2026-05-27</x:v>
+      </x:c>
+      <x:c r="E18" s="20" t="str">
+        <x:v>https://www.usitc.gov/press_room/news_release/2026/er0527_67584.htm</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="str">
+        <x:v>official trade policy</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="str">
+        <x:v>tariff continuation catalyst</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="str">
+        <x:v>primary</x:v>
+      </x:c>
       <x:c r="I18" s="2"/>
       <x:c r="J18" s="2"/>
       <x:c r="K18" s="2"/>
@@ -23596,5 +25993,8 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8293c6b1ebf4f8e"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>